<commit_message>
Add Southeast batch (6 contacts) + US Region column to outreach tracker
</commit_message>
<xml_diff>
--- a/University_Bee_Research_Contacts.xlsx
+++ b/University_Bee_Research_Contacts.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'University Contacts'!$A$1:$K$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'University Contacts'!$A$1:$L$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -46,11 +46,11 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
@@ -99,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -108,18 +108,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -485,20 +482,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -519,40 +517,45 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>US Region</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Research Focus</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Why Relevant to SaveTheHives</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Date Emailed</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Follow-up Date</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -576,32 +579,37 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>Mid-Atlantic</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>cmgrozinger@psu.edu</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>814-865-2214</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Molecular/physiological/ecological determinants of managed &amp; wild bee health; pollinator conservation</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Directs one of the largest pollinator research centers in the US, with a strong extension/outreach arm that could amplify a citizen-science mapping project.</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -621,32 +629,37 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
           <t>Use beelab.umn.edu/contact form</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>612-624-3636 (dept.)</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Honey bee social immunity, hygienic behavior, breeding for disease resistance</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>The 'Genetic Goldmine' framing (survivor colonies bred for resistance) is essentially her life's work; a major name if she engages, even briefly.</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
       <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Emeritus - personal email not published; route through lab contact form or department (entomology@umn.edu).</t>
         </is>
@@ -670,32 +683,37 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>West/Pacific</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
           <t>elnino@ucdavis.edu</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>(530) 752-1011</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Queen health, colony management, statewide extension</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>West Coast counterpart to NC State's program; UC Davis runs one of the country's top honey bee research facilities.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
     </row>
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -715,32 +733,37 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>South Central</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
           <t>juliana.rangelposada@ag.tamu.edu</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>979-845-1074</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Queen and drone reproductive biology, colony health</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Leads a major state bee program in a region with a strong feral/Africanized colony research thread already in our contact notes.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -760,32 +783,37 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
+          <t>Southeast</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
           <t>jdellis@ufl.edu</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>352-273-3924</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Colony health, feral colony/swarm removal and trapping, extension</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>HBREL runs active feral-colony removal and trapping research - closely adjacent to SaveTheHives' core mapping mission.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -805,28 +833,33 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
+          <t>Pacific Northwest</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
           <t>bhopkins@wsu.edu</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Honey bee germplasm cryopreservation, genetic diversity preservation</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Genetic-diversity/germplasm preservation work lines up directly with the 'Genetic Goldmine' survivor-genetics framing.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
       <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Succeeded Steve Sheppard (retired 2024) as program lead.</t>
         </is>
@@ -850,32 +883,37 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
           <t>johnson.5005@osu.edu</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>(330) 202-3523</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Foraging ecology, pesticide exposure</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Strong Midwest program with an active beekeeper-facing extension arm.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
     </row>
     <row r="9" ht="60" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -895,28 +933,33 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
+          <t>Northeast</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>shm33@cornell.edu</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Pesticide and pathogen impacts on pollinator health</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Northeast counterpart to Tarpy's NC State program; Dyce Lab has a large beekeeper-facing extension program to cross-promote with.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
       <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>General lab inbox is dycelab@cornell.edu if personal email bounces.</t>
         </is>
@@ -940,32 +983,37 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
+          <t>Southeast</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
           <t>ksd@uga.edu</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>706-542-2816</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Colony health, honey bee biology and behavior, IPM</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Adjacent Southeast state; UGA runs a large Master Beekeeper Program that could help cross-promote SaveTheHives.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -985,32 +1033,37 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
+          <t>Southeast</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
           <t>williams@auburn.edu</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>(334) 844-5068</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Colony health, disease and stressor interactions</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Adjacent Southeast state with a growing, well-funded bee center.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
     </row>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -1030,32 +1083,37 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
+          <t>Pacific Northwest</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
           <t>ramesh.sagili@oregonstate.edu</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>541-737-5460</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Nutrition, Varroa management, pollination</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>West Coast program with an active Master Beekeeper Program and strong grower/beekeeper outreach.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Email inferred from standard OSU firstname.lastname pattern - confirm before sending (site lists it as an obfuscated mailto).</t>
         </is>
@@ -1079,32 +1137,37 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
+          <t>Mid-Atlantic</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
           <t>dvane@umd.edu</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>301-405-3911</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Epidemiological approach to colony loss; large-scale citizen-science monitoring</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Runs the country's largest citizen-science bee health survey (the annual national Colony Loss Survey) - the closest methodological cousin to SaveTheHives on this list.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Strong candidate to lead with - his own work is citizen-science-adjacent.</t>
         </is>
@@ -1128,32 +1191,37 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
           <t>kgiven@purdue.edu</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>765-494-6747</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Mite-resistant honey bee breeding</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Directly on-thesis: breeding survivor stock for Varroa resistance.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
     </row>
     <row r="15" ht="60" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -1173,32 +1241,37 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
           <t>honeybees@msu.edu</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>(517) 884-9518</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Bacterial pathogens, honey bee medicine, risk assessment</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Trains veterinary students/professionals in honey bee medicine - an outreach channel beyond the typical beekeeping audience.</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>Lab inbox shown; address email to Dr. Milbrath by name.</t>
         </is>
@@ -1222,32 +1295,37 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
+          <t>Southeast</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
           <t>jeff.harris@msstate.edu</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>662-325-2085</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Varroa-resistant stock breeding, colony health</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Deep South program with a breeding focus that aligns closely with the Genetic Goldmine framing.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
     </row>
     <row r="17" ht="60" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
@@ -1267,32 +1345,37 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
           <t>adolezal@illinois.edu</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>217-300-6762</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Colony nutrition/stress, virus transmission between managed and wild bees</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Studies wild-managed bee interactions directly relevant to feral colony tracking.</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
     </row>
     <row r="18" ht="60" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -1312,32 +1395,37 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
+          <t>South Central</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
           <t>nkjoshi@uark.edu</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>(479) 575-3872</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Toxicology, pollinator ecology and health</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Fills a south-central US research gap in this list.</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
     </row>
     <row r="19" ht="60" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
@@ -1357,32 +1445,37 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
+          <t>Great Plains</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
           <t>jwu-smart@unl.edu</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>402-472-8696</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Pollinator health, pesticide exposure</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>Great Plains program; trained under Marla Spivak, a nice connective thread if both are contacted.</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr"/>
     </row>
     <row r="20" ht="60" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -1402,34 +1495,346 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
+          <t>Mid-Atlantic</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
           <t>mjc@vt.edu</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Honey bee foraging, recruitment, waggle-dance communication</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>Adjacent to NC/VA; foraging-ecology research could make direct use of SaveTheHives' colony location data.</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="60" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Ben Powell</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Coordinator, Apiculture and Pollinator Program</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Clemson University</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Southeast</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>bpowel2@clemson.edu</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>843-662-3526</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Extension support for SC beekeepers, pollinator conservation outreach</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Neighboring state extension program (SC) with an active beekeeper-facing newsletter (CAPPings) that could carry a SaveTheHives mention statewide.</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22" ht="60" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Jennifer Tsuruda</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Assistant Professor; Apiculture Extension Specialist</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>University of Tennessee, Knoxville</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Southeast</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>jennifer.tsuruda@utk.edu</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Honey bee health and management, pollination, beekeeper education</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Runs the TN Master Beekeeping Program (previously at Clemson) - a large existing beekeeper network one door down from NC.</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Email inferred from standard UTK firstname.lastname pattern - confirm before sending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="60" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Morgan Christman</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Pollinator Ecology</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>LSU AgCenter / Louisiana State University</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Southeast</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>MChristman@agcenter.lsu.edu</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Pollinator ecology and conservation; building baseline pollinator/native bee data for Louisiana</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Brand-new program (2025) actively building citizen-science partnerships (a Louisiana Bumble Bee Atlas) - likely receptive to a sister citizen-science project.</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24" ht="60" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Yong-Lak Park</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Professor of Entomology</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>West Virginia University</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Mid-Atlantic</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Yong-Lak.Park@mail.wvu.edu</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>(304) 293-2882</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Integrated pest management, pollination ecology of solitary/wild bees, geospatial/remote-sensing methods</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>His geospatial/remote-sensing angle on wild bee ecology is a natural methodological conversation with a location-mapping app.</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Focus is broader than honey bees specifically (solitary bees, IPM) - tailor the relevance line accordingly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="60" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Rahman Tashakkori</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Lowe's Distinguished Professor of Computer Science; PI, AppMAIS Project</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Appalachian State University</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Southeast</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>tashakkorir@appstate.edu</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>(828) 262-7009</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Honey bee health monitoring systems (hive sensors, data science, AI) - the AppMAIS/Beemon project</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Closest technical cousin on this whole list: an NC-based (Boone) honeybee data/monitoring project. Strong potential collaborator, not just an outreach target - worth a more tailored note than the standard boilerplate.</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Computer Science, not entomology/biology - AppMAIS is the hook, not a traditional bee lab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="60" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Amy Vu</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>State Specialized Extension Agent II, Apiculture</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>University of Florida (Honey Bee Research &amp; Extension Lab)</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Southeast</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>amy.vu@ufl.edu</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Beekeeper education, UF Master Beekeeper Program, Bee College, extension outreach</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Runs UF's beekeeper-facing extension/outreach programs (Bee College, Master Beekeeper Program) - a second, extension-focused UF contact alongside Dr. Ellis's research-focused one.</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Same institution as Jamie Ellis (already on this list) but a distinct extension-facing role - fine to contact both.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K20"/>
-  <dataValidations count="1">
-    <dataValidation sqref="H2:H20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <autoFilter ref="A1:L26"/>
+  <dataValidations count="2">
+    <dataValidation sqref="I2:I26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Contacted,Emailed - Awaiting Reply,Replied,Call/Meeting Scheduled,Declined,No Longer Pursuing"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Northeast,Mid-Atlantic,Southeast,Midwest,Great Plains,South Central,Mountain West,Pacific Northwest,West/Pacific"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1457,97 +1862,97 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>How to use this template</t>
         </is>
       </c>
     </row>
     <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Copy the Subject and Body below into Gmail for each contact. Fill in the bracketed placeholders using that contact's row on the "University Contacts" tab — Name, Institution, and especially the "Why Relevant to SaveTheHives" column, which is written so it can drop almost directly into [RELEVANCE SENTENCE]. Keep the rest as-is; it's deliberately short. After sending, update Status and Date Emailed on the University Contacts tab.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Placeholders</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>[FIRST NAME]</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Contact's first name (e.g. Christina)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>[LAST NAME]</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Contact's last name, as it appears after "Dr." (e.g. Grozinger)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>[INSTITUTION]</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>University name (e.g. Penn State University)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>[RELEVANCE SENTENCE]</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>One sentence tying their specific research to SaveTheHives — start from the "Why Relevant" column and adjust the wording so it reads naturally in a sentence.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Subject</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Wild honeybee colony mapping project — thought of your work at [INSTITUTION]</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Body</t>
         </is>
       </c>
     </row>
     <row r="16" ht="430" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>Hi Dr. [LAST NAME],
 My name is Ronnie Bouchon, and I run SaveTheHives (savethehives.org), a free citizen-science app for mapping wild/feral honeybee colonies — tree cavities, structures, ground nests, wherever people find them. The app currently has 1,150+ historical hive records live on the map (many concentrated around the NC Triangle), and volunteers can log new colonies or simply re-verify ("Validate") an existing one.
@@ -1578,7 +1983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1592,70 +1997,87 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr"/>
+      <c r="A2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Purpose: track outreach to university honey bee / apiculture research programs that may want to know about savethehives.org.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr"/>
+      <c r="A4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>How to use this sheet:</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>1. Update the Status dropdown (column H) as you email each contact: Not Contacted -&gt; Emailed - Awaiting Reply -&gt; Replied / Call-Meeting Scheduled / Declined / No Longer Pursuing.</t>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>1. Update the Status dropdown (column I) as you email each contact: Not Contacted -&gt; Emailed - Awaiting Reply -&gt; Replied / Call-Meeting Scheduled / Declined / No Longer Pursuing.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>2. Fill in Date Emailed (column I) when you send the first email.</t>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>2. Fill in Date Emailed (column J) when you send the first email.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>3. Set a Follow-up Date (column J) — a reasonable rule of thumb is 2-3 weeks after the initial email if there's been no reply.</t>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>3. Set a Follow-up Date (column K) — a reasonable rule of thumb is 2-3 weeks after the initial email if there's been no reply.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>4. Use Notes (column K) for anything short and specific: what they said, a call summary, a second contact they mentioned, etc.</t>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>4. Use Notes (column L) for anything short and specific: what they said, a call summary, a second contact they mentioned, etc.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr"/>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>5. US Region (column D) is a dropdown too, in case you add more contacts later and want the categories to stay consistent: Northeast, Mid-Atlantic, Southeast, Midwest, Great Plains, South Central, Mountain West, Pacific Northwest, West/Pacific.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Batches so far: Batch 1 (Jul 25 2026) — 19 contacts, national spread. Batch 2 (Jul 25 2026) — 6 contacts, Southeast-focused (Clemson, UT Knoxville, LSU, WVU, Appalachian State, UF Extension).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>This list is separate from KEY_PEOPLE_CONTACTS.md in the project repo, which tracks advisors and leads already in motion (Tarpy, Delaney, Wake County Beekeepers, Julia Mahood, etc.). Once outreach starts here, it's worth mirroring status updates into that file too so both stay in sync.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>All contacts are faculty PIs / program directors — no grad students or postdocs included in this pass, per your instruction to keep this to PI-level contacts for now.</t>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>All contacts are faculty PIs / program directors / lead specialists — no grad students or postdocs included in either batch, per your instruction to keep this to PI-level contacts.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Seeley, Tarpy, Delaney to university contacts tracker
</commit_message>
<xml_diff>
--- a/University_Bee_Research_Contacts.xlsx
+++ b/University_Bee_Research_Contacts.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'University Contacts'!$A$1:$L$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'University Contacts'!$A$1:$L$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -59,7 +59,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -70,6 +70,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F5A623"/>
         <bgColor rgb="00F5A623"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3D6"/>
+        <bgColor rgb="00FFF3D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -99,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -117,6 +123,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -482,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -561,199 +570,207 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Dr. Christina Grozinger</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Professor of Entomology; Director, Center for Pollinator Research</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Penn State University</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
+    <row r="2" ht="70" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Dr. Thomas D. Seeley</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>Horace White Professor Emeritus in Biology, Dept. of Neurobiology and Behavior</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>Cornell University</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>Northeast</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>tds5@cornell.edu</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>(607) 279-5498</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>Swarm intelligence and collective decision-making in honey bee colonies; wild/feral colony survival without Varroa treatment (Arnot Forest, NY, ongoing since 2011)</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>The scientific foundation of the whole 'Genetic Goldmine' framing: his Arnot Forest feral-colony study is the original long-running demonstration that untreated wild colonies persist and adapt to Varroa. Author of Honeybee Democracy and The Lives of Bees. Already a co-author with Tarpy and Delaney (Seeley, Tarpy, Griffin, Carcione, Delaney 2015, Apidologie) on wild colony genetic structure - arguably the single most on-thesis name on this whole list.</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="J2" s="9" t="inlineStr"/>
+      <c r="K2" s="9" t="inlineStr"/>
+      <c r="L2" s="9" t="inlineStr">
+        <is>
+          <t>Extremely high-value contact - worth a personally written email referencing the 2015 Apidologie paper rather than the generic boilerplate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="70" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Dr. David R. Tarpy</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>University Scholar Professor &amp; Extension Apiculturist, Dept. of Applied Ecology</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>NC State University</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Southeast</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>drtarpy@ncsu.edu</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr"/>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>Behavioral ecology of honey bee queens (polyandry, intracolony genetic diversity), social immunity, IPM, queen reproductive quality</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>Named scientific advisor on SaveTheHives' 'Genetic Goldmine' framing since the Jul 21 2026 lunch meeting - reviewed and approved all 5 questions on the language handout. Helped get the original savethehives.com press coverage in 2008.</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>Confirmed - Advisor</t>
+        </is>
+      </c>
+      <c r="J3" s="9" t="inlineStr"/>
+      <c r="K3" s="9" t="inlineStr"/>
+      <c r="L3" s="9" t="inlineStr">
+        <is>
+          <t>Already actively engaged - not part of the cold-outreach batches below. Included here so this list reads as complete when shared with him. See MEETING_NOTES_2026-07-21_Tarpy.md for full context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="70" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Dr. Debbie Delaney</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Charles P. Townsend Family Professor of Pollinator Science, Dept. of Entomology &amp; Wildlife Ecology</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>University of Delaware</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Mid-Atlantic</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>cmgrozinger@psu.edu</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>814-865-2214</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Molecular/physiological/ecological determinants of managed &amp; wild bee health; pollinator conservation</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Directs one of the largest pollinator research centers in the US, with a strong extension/outreach arm that could amplify a citizen-science mapping project.</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3" ht="60" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Dr. Marla Spivak</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Professor Emeritus (MacArthur Fellow); Bee Lab</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>University of Minnesota</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Midwest</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Use beelab.umn.edu/contact form</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>612-624-3636 (dept.)</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Honey bee social immunity, hygienic behavior, breeding for disease resistance</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>The 'Genetic Goldmine' framing (survivor colonies bred for resistance) is essentially her life's work; a major name if she engages, even briefly.</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>Emeritus - personal email not published; route through lab contact form or department (entomology@umn.edu).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Dr. Elina Nino</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Professor of Cooperative Extension, Apiculture</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>UC Davis (Harry H. Laidlaw Jr. Honey Bee Research Facility)</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>West/Pacific</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>elnino@ucdavis.edu</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>(530) 752-1011</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Queen health, colony management, statewide extension</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>West Coast counterpart to NC State's program; UC Davis runs one of the country's top honey bee research facilities.</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>dadelane@udel.edu</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>302-831-8883</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>Evolutionary biology and population genetics of honey bees, benefits of polyandry on colony health, IPM</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>Her UD faculty page lists savethehives.com as one of her own resource links - she was directly involved with the original 2008-era project alongside Tarpy. Co-author with Tarpy and Seeley on the 2015 Apidologie survivor-colony genetics paper - directly on-thesis for the Genetic Goldmine framing.</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>Emailed - Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr"/>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>Reintroduction email sent 2026-07-25 (see delaney-email.html / KEY_PEOPLE_CONTACTS.md). Not part of the cold-outreach batches below - included here so this list reads as complete when shared with Tarpy.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Dr. Juliana Rangel</t>
+          <t>Dr. Christina Grozinger</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Associate Professor of Apiculture</t>
+          <t>Professor of Entomology; Director, Center for Pollinator Research</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Texas A&amp;M University</t>
+          <t>Penn State University</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>South Central</t>
+          <t>Mid-Atlantic</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>juliana.rangelposada@ag.tamu.edu</t>
+          <t>cmgrozinger@psu.edu</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>979-845-1074</t>
+          <t>814-865-2214</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Queen and drone reproductive biology, colony health</t>
+          <t>Molecular/physiological/ecological determinants of managed &amp; wild bee health; pollinator conservation</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Leads a major state bee program in a region with a strong feral/Africanized colony research thread already in our contact notes.</t>
+          <t>Directs one of the largest pollinator research centers in the US, with a strong extension/outreach arm that could amplify a citizen-science mapping project.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -761,49 +778,49 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="n"/>
+      <c r="K5" s="2" t="n"/>
+      <c r="L5" s="2" t="n"/>
     </row>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Dr. Jamie Ellis</t>
+          <t>Dr. Marla Spivak</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Gahan Endowed Professor; Director, Honey Bee Research &amp; Extension Lab</t>
+          <t>Professor Emeritus (MacArthur Fellow); Bee Lab</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>University of Florida</t>
+          <t>University of Minnesota</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>jdellis@ufl.edu</t>
+          <t>Use beelab.umn.edu/contact form</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>352-273-3924</t>
+          <t>612-624-3636 (dept.)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Colony health, feral colony/swarm removal and trapping, extension</t>
+          <t>Honey bee social immunity, hygienic behavior, breeding for disease resistance</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>HBREL runs active feral-colony removal and trapping research - closely adjacent to SaveTheHives' core mapping mission.</t>
+          <t>The 'Genetic Goldmine' framing (survivor colonies bred for resistance) is essentially her life's work; a major name if she engages, even briefly.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -811,45 +828,53 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="2" t="n"/>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Emeritus - personal email not published; route through lab contact form or department (entomology@umn.edu).</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Dr. Brandon Hopkins</t>
+          <t>Dr. Elina Nino</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Thurber Endowed Distinguished Professor of Pollinator Ecology</t>
+          <t>Professor of Cooperative Extension, Apiculture</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Washington State University</t>
+          <t>UC Davis (Harry H. Laidlaw Jr. Honey Bee Research Facility)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Pacific Northwest</t>
+          <t>West/Pacific</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>bhopkins@wsu.edu</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr"/>
+          <t>elnino@ucdavis.edu</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>(530) 752-1011</t>
+        </is>
+      </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Honey bee germplasm cryopreservation, genetic diversity preservation</t>
+          <t>Queen health, colony management, statewide extension</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Genetic-diversity/germplasm preservation work lines up directly with the 'Genetic Goldmine' survivor-genetics framing.</t>
+          <t>West Coast counterpart to NC State's program; UC Davis runs one of the country's top honey bee research facilities.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -857,53 +882,49 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>Succeeded Steve Sheppard (retired 2024) as program lead.</t>
-        </is>
-      </c>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="2" t="n"/>
     </row>
     <row r="8" ht="60" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Dr. Reed Johnson</t>
+          <t>Dr. Juliana Rangel</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Associate Professor, Bee Lab</t>
+          <t>Associate Professor of Apiculture</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Ohio State University</t>
+          <t>Texas A&amp;M University</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>South Central</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>johnson.5005@osu.edu</t>
+          <t>juliana.rangelposada@ag.tamu.edu</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>(330) 202-3523</t>
+          <t>979-845-1074</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Foraging ecology, pesticide exposure</t>
+          <t>Queen and drone reproductive biology, colony health</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Strong Midwest program with an active beekeeper-facing extension arm.</t>
+          <t>Leads a major state bee program in a region with a strong feral/Africanized colony research thread already in our contact notes.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -911,45 +932,49 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="n"/>
+      <c r="K8" s="2" t="n"/>
+      <c r="L8" s="2" t="n"/>
     </row>
     <row r="9" ht="60" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Dr. Scott McArt</t>
+          <t>Dr. Jamie Ellis</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Associate Professor of Pollinator Health; Director, Dyce Lab for Honey Bee Studies</t>
+          <t>Gahan Endowed Professor; Director, Honey Bee Research &amp; Extension Lab</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Cornell University</t>
+          <t>University of Florida</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Northeast</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>shm33@cornell.edu</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr"/>
+          <t>jdellis@ufl.edu</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>352-273-3924</t>
+        </is>
+      </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Pesticide and pathogen impacts on pollinator health</t>
+          <t>Colony health, feral colony/swarm removal and trapping, extension</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Northeast counterpart to Tarpy's NC State program; Dyce Lab has a large beekeeper-facing extension program to cross-promote with.</t>
+          <t>HBREL runs active feral-colony removal and trapping research - closely adjacent to SaveTheHives' core mapping mission.</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -957,53 +982,45 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>General lab inbox is dycelab@cornell.edu if personal email bounces.</t>
-        </is>
-      </c>
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" s="2" t="n"/>
+      <c r="L9" s="2" t="n"/>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Dr. Keith Delaplane</t>
+          <t>Dr. Brandon Hopkins</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Professor Emeritus; Director, UGA Bee Program</t>
+          <t>Thurber Endowed Distinguished Professor of Pollinator Ecology</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>University of Georgia</t>
+          <t>Washington State University</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Pacific Northwest</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>ksd@uga.edu</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>706-542-2816</t>
-        </is>
-      </c>
+          <t>bhopkins@wsu.edu</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Colony health, honey bee biology and behavior, IPM</t>
+          <t>Honey bee germplasm cryopreservation, genetic diversity preservation</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Adjacent Southeast state; UGA runs a large Master Beekeeper Program that could help cross-promote SaveTheHives.</t>
+          <t>Genetic-diversity/germplasm preservation work lines up directly with the 'Genetic Goldmine' survivor-genetics framing.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1011,49 +1028,53 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="n"/>
+      <c r="K10" s="2" t="n"/>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Succeeded Steve Sheppard (retired 2024) as program lead.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Dr. Geoff Williams</t>
+          <t>Dr. Reed Johnson</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Associate Professor; Director, Bee Center</t>
+          <t>Associate Professor, Bee Lab</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Auburn University</t>
+          <t>Ohio State University</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>williams@auburn.edu</t>
+          <t>johnson.5005@osu.edu</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>(334) 844-5068</t>
+          <t>(330) 202-3523</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Colony health, disease and stressor interactions</t>
+          <t>Foraging ecology, pesticide exposure</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Adjacent Southeast state with a growing, well-funded bee center.</t>
+          <t>Strong Midwest program with an active beekeeper-facing extension arm.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1061,49 +1082,45 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="n"/>
+      <c r="K11" s="2" t="n"/>
+      <c r="L11" s="2" t="n"/>
     </row>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Dr. Ramesh Sagili</t>
+          <t>Dr. Scott McArt</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Professor of Apiculture, Honey Bee Lab</t>
+          <t>Associate Professor of Pollinator Health; Director, Dyce Lab for Honey Bee Studies</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Oregon State University</t>
+          <t>Cornell University</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Pacific Northwest</t>
+          <t>Northeast</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>ramesh.sagili@oregonstate.edu</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>541-737-5460</t>
-        </is>
-      </c>
+          <t>shm33@cornell.edu</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n"/>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Nutrition, Varroa management, pollination</t>
+          <t>Pesticide and pathogen impacts on pollinator health</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>West Coast program with an active Master Beekeeper Program and strong grower/beekeeper outreach.</t>
+          <t>Northeast counterpart to Tarpy's NC State program; Dyce Lab has a large beekeeper-facing extension program to cross-promote with.</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1111,53 +1128,53 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="n"/>
+      <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Email inferred from standard OSU firstname.lastname pattern - confirm before sending (site lists it as an obfuscated mailto).</t>
+          <t>General lab inbox is dycelab@cornell.edu if personal email bounces.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="60" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Dr. Dennis vanEngelsdorp</t>
+          <t>Dr. Keith Delaplane</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Professor; Chief Scientist, Bee Informed Partnership</t>
+          <t>Professor Emeritus; Director, UGA Bee Program</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>University of Maryland</t>
+          <t>University of Georgia</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Mid-Atlantic</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>dvane@umd.edu</t>
+          <t>ksd@uga.edu</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>301-405-3911</t>
+          <t>706-542-2816</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Epidemiological approach to colony loss; large-scale citizen-science monitoring</t>
+          <t>Colony health, honey bee biology and behavior, IPM</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Runs the country's largest citizen-science bee health survey (the annual national Colony Loss Survey) - the closest methodological cousin to SaveTheHives on this list.</t>
+          <t>Adjacent Southeast state; UGA runs a large Master Beekeeper Program that could help cross-promote SaveTheHives.</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1165,53 +1182,49 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>Strong candidate to lead with - his own work is citizen-science-adjacent.</t>
-        </is>
-      </c>
+      <c r="J13" s="2" t="n"/>
+      <c r="K13" s="2" t="n"/>
+      <c r="L13" s="2" t="n"/>
     </row>
     <row r="14" ht="60" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Krispn Given</t>
+          <t>Dr. Geoff Williams</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Senior Apiculture Specialist, Honey Bee Breeding Program</t>
+          <t>Associate Professor; Director, Bee Center</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Purdue University</t>
+          <t>Auburn University</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>kgiven@purdue.edu</t>
+          <t>williams@auburn.edu</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>765-494-6747</t>
+          <t>(334) 844-5068</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Mite-resistant honey bee breeding</t>
+          <t>Colony health, disease and stressor interactions</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Directly on-thesis: breeding survivor stock for Varroa resistance.</t>
+          <t>Adjacent Southeast state with a growing, well-funded bee center.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1219,49 +1232,49 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="n"/>
+      <c r="K14" s="2" t="n"/>
+      <c r="L14" s="2" t="n"/>
     </row>
     <row r="15" ht="60" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Dr. Meghan Milbrath</t>
+          <t>Dr. Ramesh Sagili</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Academic Specialist; Coordinator, Michigan Pollinator Initiative</t>
+          <t>Professor of Apiculture, Honey Bee Lab</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Michigan State University</t>
+          <t>Oregon State University</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>Pacific Northwest</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>honeybees@msu.edu</t>
+          <t>ramesh.sagili@oregonstate.edu</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>(517) 884-9518</t>
+          <t>541-737-5460</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Bacterial pathogens, honey bee medicine, risk assessment</t>
+          <t>Nutrition, Varroa management, pollination</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Trains veterinary students/professionals in honey bee medicine - an outreach channel beyond the typical beekeeping audience.</t>
+          <t>West Coast program with an active Master Beekeeper Program and strong grower/beekeeper outreach.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1269,53 +1282,53 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="n"/>
+      <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Lab inbox shown; address email to Dr. Milbrath by name.</t>
+          <t>Email inferred from standard OSU firstname.lastname pattern - confirm before sending (site lists it as an obfuscated mailto).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="60" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Dr. Jeff Harris</t>
+          <t>Dr. Dennis vanEngelsdorp</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Associate Professor, Apiculture Extension Specialist</t>
+          <t>Professor; Chief Scientist, Bee Informed Partnership</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Mississippi State University</t>
+          <t>University of Maryland</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Mid-Atlantic</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>jeff.harris@msstate.edu</t>
+          <t>dvane@umd.edu</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>662-325-2085</t>
+          <t>301-405-3911</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Varroa-resistant stock breeding, colony health</t>
+          <t>Epidemiological approach to colony loss; large-scale citizen-science monitoring</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Deep South program with a breeding focus that aligns closely with the Genetic Goldmine framing.</t>
+          <t>Runs the country's largest citizen-science bee health survey (the annual national Colony Loss Survey) - the closest methodological cousin to SaveTheHives on this list.</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1323,24 +1336,28 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="n"/>
+      <c r="K16" s="2" t="n"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Strong candidate to lead with - his own work is citizen-science-adjacent.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="60" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Dr. Adam Dolezal</t>
+          <t>Krispn Given</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Associate Professor, Dolezal Bee Research Lab</t>
+          <t>Senior Apiculture Specialist, Honey Bee Breeding Program</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>University of Illinois Urbana-Champaign</t>
+          <t>Purdue University</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1350,22 +1367,22 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>adolezal@illinois.edu</t>
+          <t>kgiven@purdue.edu</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>217-300-6762</t>
+          <t>765-494-6747</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Colony nutrition/stress, virus transmission between managed and wild bees</t>
+          <t>Mite-resistant honey bee breeding</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Studies wild-managed bee interactions directly relevant to feral colony tracking.</t>
+          <t>Directly on-thesis: breeding survivor stock for Varroa resistance.</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1373,49 +1390,49 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr"/>
-      <c r="K17" s="2" t="inlineStr"/>
-      <c r="L17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="n"/>
+      <c r="K17" s="2" t="n"/>
+      <c r="L17" s="2" t="n"/>
     </row>
     <row r="18" ht="60" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Dr. Neelendra Joshi</t>
+          <t>Dr. Meghan Milbrath</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Professor, Apiculture &amp; Pollinator Health</t>
+          <t>Academic Specialist; Coordinator, Michigan Pollinator Initiative</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>University of Arkansas</t>
+          <t>Michigan State University</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>South Central</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>nkjoshi@uark.edu</t>
+          <t>honeybees@msu.edu</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>(479) 575-3872</t>
+          <t>(517) 884-9518</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Toxicology, pollinator ecology and health</t>
+          <t>Bacterial pathogens, honey bee medicine, risk assessment</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Fills a south-central US research gap in this list.</t>
+          <t>Trains veterinary students/professionals in honey bee medicine - an outreach channel beyond the typical beekeeping audience.</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1423,49 +1440,53 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr"/>
-      <c r="K18" s="2" t="inlineStr"/>
-      <c r="L18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="n"/>
+      <c r="K18" s="2" t="n"/>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Lab inbox shown; address email to Dr. Milbrath by name.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="60" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Dr. Judy Wu-Smart</t>
+          <t>Dr. Jeff Harris</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Associate Professor, Bee Lab</t>
+          <t>Associate Professor, Apiculture Extension Specialist</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>University of Nebraska-Lincoln</t>
+          <t>Mississippi State University</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Great Plains</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>jwu-smart@unl.edu</t>
+          <t>jeff.harris@msstate.edu</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>402-472-8696</t>
+          <t>662-325-2085</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Pollinator health, pesticide exposure</t>
+          <t>Varroa-resistant stock breeding, colony health</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Great Plains program; trained under Marla Spivak, a nice connective thread if both are contacted.</t>
+          <t>Deep South program with a breeding focus that aligns closely with the Genetic Goldmine framing.</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -1473,45 +1494,49 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr"/>
-      <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="n"/>
+      <c r="K19" s="2" t="n"/>
+      <c r="L19" s="2" t="n"/>
     </row>
     <row r="20" ht="60" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Dr. Margaret Couvillon</t>
+          <t>Dr. Adam Dolezal</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Associate Professor, Pollinator Biology and Ecology</t>
+          <t>Associate Professor, Dolezal Bee Research Lab</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Virginia Tech</t>
+          <t>University of Illinois Urbana-Champaign</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Mid-Atlantic</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>mjc@vt.edu</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr"/>
+          <t>adolezal@illinois.edu</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>217-300-6762</t>
+        </is>
+      </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Honey bee foraging, recruitment, waggle-dance communication</t>
+          <t>Colony nutrition/stress, virus transmission between managed and wild bees</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Adjacent to NC/VA; foraging-ecology research could make direct use of SaveTheHives' colony location data.</t>
+          <t>Studies wild-managed bee interactions directly relevant to feral colony tracking.</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -1519,49 +1544,49 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr"/>
-      <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="n"/>
+      <c r="K20" s="2" t="n"/>
+      <c r="L20" s="2" t="n"/>
     </row>
     <row r="21" ht="60" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Ben Powell</t>
+          <t>Dr. Neelendra Joshi</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Coordinator, Apiculture and Pollinator Program</t>
+          <t>Professor, Apiculture &amp; Pollinator Health</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Clemson University</t>
+          <t>University of Arkansas</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>South Central</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>bpowel2@clemson.edu</t>
+          <t>nkjoshi@uark.edu</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>843-662-3526</t>
+          <t>(479) 575-3872</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Extension support for SC beekeepers, pollinator conservation outreach</t>
+          <t>Toxicology, pollinator ecology and health</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Neighboring state extension program (SC) with an active beekeeper-facing newsletter (CAPPings) that could carry a SaveTheHives mention statewide.</t>
+          <t>Fills a south-central US research gap in this list.</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -1569,45 +1594,49 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr"/>
-      <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="n"/>
+      <c r="K21" s="2" t="n"/>
+      <c r="L21" s="2" t="n"/>
     </row>
     <row r="22" ht="60" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Dr. Jennifer Tsuruda</t>
+          <t>Dr. Judy Wu-Smart</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor; Apiculture Extension Specialist</t>
+          <t>Associate Professor, Bee Lab</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>University of Tennessee, Knoxville</t>
+          <t>University of Nebraska-Lincoln</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Great Plains</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>jennifer.tsuruda@utk.edu</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr"/>
+          <t>jwu-smart@unl.edu</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>402-472-8696</t>
+        </is>
+      </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Honey bee health and management, pollination, beekeeper education</t>
+          <t>Pollinator health, pesticide exposure</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Runs the TN Master Beekeeping Program (previously at Clemson) - a large existing beekeeper network one door down from NC.</t>
+          <t>Great Plains program; trained under Marla Spivak, a nice connective thread if both are contacted.</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1615,49 +1644,45 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>Email inferred from standard UTK firstname.lastname pattern - confirm before sending.</t>
-        </is>
-      </c>
+      <c r="J22" s="2" t="n"/>
+      <c r="K22" s="2" t="n"/>
+      <c r="L22" s="2" t="n"/>
     </row>
     <row r="23" ht="60" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Dr. Morgan Christman</t>
+          <t>Dr. Margaret Couvillon</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Pollinator Ecology</t>
+          <t>Associate Professor, Pollinator Biology and Ecology</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>LSU AgCenter / Louisiana State University</t>
+          <t>Virginia Tech</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Mid-Atlantic</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>MChristman@agcenter.lsu.edu</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr"/>
+          <t>mjc@vt.edu</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Pollinator ecology and conservation; building baseline pollinator/native bee data for Louisiana</t>
+          <t>Honey bee foraging, recruitment, waggle-dance communication</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Brand-new program (2025) actively building citizen-science partnerships (a Louisiana Bumble Bee Atlas) - likely receptive to a sister citizen-science project.</t>
+          <t>Adjacent to NC/VA; foraging-ecology research could make direct use of SaveTheHives' colony location data.</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -1665,49 +1690,49 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr"/>
-      <c r="K23" s="2" t="inlineStr"/>
-      <c r="L23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="n"/>
+      <c r="K23" s="2" t="n"/>
+      <c r="L23" s="2" t="n"/>
     </row>
     <row r="24" ht="60" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Dr. Yong-Lak Park</t>
+          <t>Ben Powell</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Professor of Entomology</t>
+          <t>Coordinator, Apiculture and Pollinator Program</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>West Virginia University</t>
+          <t>Clemson University</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Mid-Atlantic</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Yong-Lak.Park@mail.wvu.edu</t>
+          <t>bpowel2@clemson.edu</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>(304) 293-2882</t>
+          <t>843-662-3526</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Integrated pest management, pollination ecology of solitary/wild bees, geospatial/remote-sensing methods</t>
+          <t>Extension support for SC beekeepers, pollinator conservation outreach</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>His geospatial/remote-sensing angle on wild bee ecology is a natural methodological conversation with a location-mapping app.</t>
+          <t>Neighboring state extension program (SC) with an active beekeeper-facing newsletter (CAPPings) that could carry a SaveTheHives mention statewide.</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1715,28 +1740,24 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr"/>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>Focus is broader than honey bees specifically (solitary bees, IPM) - tailor the relevance line accordingly.</t>
-        </is>
-      </c>
+      <c r="J24" s="2" t="n"/>
+      <c r="K24" s="2" t="n"/>
+      <c r="L24" s="2" t="n"/>
     </row>
     <row r="25" ht="60" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Dr. Rahman Tashakkori</t>
+          <t>Dr. Jennifer Tsuruda</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Lowe's Distinguished Professor of Computer Science; PI, AppMAIS Project</t>
+          <t>Assistant Professor; Apiculture Extension Specialist</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Appalachian State University</t>
+          <t>University of Tennessee, Knoxville</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1746,22 +1767,18 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>tashakkorir@appstate.edu</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>(828) 262-7009</t>
-        </is>
-      </c>
+          <t>jennifer.tsuruda@utk.edu</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Honey bee health monitoring systems (hive sensors, data science, AI) - the AppMAIS/Beemon project</t>
+          <t>Honey bee health and management, pollination, beekeeper education</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Closest technical cousin on this whole list: an NC-based (Boone) honeybee data/monitoring project. Strong potential collaborator, not just an outreach target - worth a more tailored note than the standard boilerplate.</t>
+          <t>Runs the TN Master Beekeeping Program (previously at Clemson) - a large existing beekeeper network one door down from NC.</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -1769,71 +1786,225 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="n"/>
+      <c r="K25" s="2" t="n"/>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Computer Science, not entomology/biology - AppMAIS is the hook, not a traditional bee lab.</t>
+          <t>Email inferred from standard UTK firstname.lastname pattern - confirm before sending.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="60" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t>Dr. Morgan Christman</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Pollinator Ecology</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>LSU AgCenter / Louisiana State University</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Southeast</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>MChristman@agcenter.lsu.edu</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Pollinator ecology and conservation; building baseline pollinator/native bee data for Louisiana</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Brand-new program (2025) actively building citizen-science partnerships (a Louisiana Bumble Bee Atlas) - likely receptive to a sister citizen-science project.</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="n"/>
+      <c r="K26" s="2" t="n"/>
+      <c r="L26" s="2" t="n"/>
+    </row>
+    <row r="27" ht="60" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Yong-Lak Park</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Professor of Entomology</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>West Virginia University</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Mid-Atlantic</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Yong-Lak.Park@mail.wvu.edu</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>(304) 293-2882</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Integrated pest management, pollination ecology of solitary/wild bees, geospatial/remote-sensing methods</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>His geospatial/remote-sensing angle on wild bee ecology is a natural methodological conversation with a location-mapping app.</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="n"/>
+      <c r="K27" s="2" t="n"/>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>Focus is broader than honey bees specifically (solitary bees, IPM) - tailor the relevance line accordingly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="60" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Rahman Tashakkori</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Lowe's Distinguished Professor of Computer Science; PI, AppMAIS Project</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Appalachian State University</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Southeast</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>tashakkorir@appstate.edu</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>(828) 262-7009</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Honey bee health monitoring systems (hive sensors, data science, AI) - the AppMAIS/Beemon project</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Closest technical cousin on this whole list: an NC-based (Boone) honeybee data/monitoring project. Strong potential collaborator, not just an outreach target - worth a more tailored note than the standard boilerplate.</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="n"/>
+      <c r="K28" s="2" t="n"/>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Computer Science, not entomology/biology - AppMAIS is the hook, not a traditional bee lab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="60" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>Amy Vu</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>State Specialized Extension Agent II, Apiculture</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>University of Florida (Honey Bee Research &amp; Extension Lab)</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Southeast</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>amy.vu@ufl.edu</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr"/>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>Beekeeper education, UF Master Beekeeper Program, Bee College, extension outreach</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>Runs UF's beekeeper-facing extension/outreach programs (Bee College, Master Beekeeper Program) - a second, extension-focused UF contact alongside Dr. Ellis's research-focused one.</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr"/>
-      <c r="K26" s="2" t="inlineStr"/>
-      <c r="L26" s="2" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="n"/>
+      <c r="K29" s="2" t="n"/>
+      <c r="L29" s="2" t="inlineStr">
         <is>
           <t>Same institution as Jamie Ellis (already on this list) but a distinct extension-facing role - fine to contact both.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L26"/>
+  <autoFilter ref="A1:L29"/>
   <dataValidations count="2">
-    <dataValidation sqref="I2:I26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Not Contacted,Emailed - Awaiting Reply,Replied,Call/Meeting Scheduled,Declined,No Longer Pursuing"</formula1>
+    <dataValidation sqref="I2:I29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Not Contacted,Emailed - Awaiting Reply,Replied,Call/Meeting Scheduled,Declined,No Longer Pursuing,Confirmed - Advisor"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Northeast,Mid-Atlantic,Southeast,Midwest,Great Plains,South Central,Mountain West,Pacific Northwest,West/Pacific"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1983,7 +2154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -2012,52 +2183,52 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>How to use this sheet:</t>
+          <t>Rows 2-4 (highlighted): Dr. Thomas Seeley (Cornell), Dr. David Tarpy (NC State), and Dr. Debbie Delaney (U Delaware) — the three researchers already central to this project. Tarpy is a confirmed named advisor; Delaney was emailed 2026-07-25 and is awaiting reply; Seeley is the scientific originator of the wild-colony-survival research this project's framing is built on, and has co-authored with the other two. They're listed first, separately from the batches below, so the sheet reads as complete at a glance if shared with Tarpy.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>1. Update the Status dropdown (column I) as you email each contact: Not Contacted -&gt; Emailed - Awaiting Reply -&gt; Replied / Call-Meeting Scheduled / Declined / No Longer Pursuing.</t>
-        </is>
-      </c>
+      <c r="A6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>2. Fill in Date Emailed (column J) when you send the first email.</t>
+          <t>How to use this sheet:</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>3. Set a Follow-up Date (column K) — a reasonable rule of thumb is 2-3 weeks after the initial email if there's been no reply.</t>
+          <t>1. Update the Status dropdown (column I) as you email each contact: Not Contacted -&gt; Emailed - Awaiting Reply -&gt; Replied / Call-Meeting Scheduled / Declined / No Longer Pursuing / Confirmed - Advisor.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>4. Use Notes (column L) for anything short and specific: what they said, a call summary, a second contact they mentioned, etc.</t>
+          <t>2. Fill in Date Emailed (column J) when you send the first email.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>5. US Region (column D) is a dropdown too, in case you add more contacts later and want the categories to stay consistent: Northeast, Mid-Atlantic, Southeast, Midwest, Great Plains, South Central, Mountain West, Pacific Northwest, West/Pacific.</t>
+          <t>3. Set a Follow-up Date (column K) — a reasonable rule of thumb is 2-3 weeks after the initial email if there's been no reply.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr"/>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>4. Use Notes (column L) for anything short and specific: what they said, a call summary, a second contact they mentioned, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Batches so far: Batch 1 (Jul 25 2026) — 19 contacts, national spread. Batch 2 (Jul 25 2026) — 6 contacts, Southeast-focused (Clemson, UT Knoxville, LSU, WVU, Appalachian State, UF Extension).</t>
+          <t>5. US Region (column D) is a dropdown too, in case you add more contacts later and want the categories to stay consistent: Northeast, Mid-Atlantic, Southeast, Midwest, Great Plains, South Central, Mountain West, Pacific Northwest, West/Pacific.</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2238,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>This list is separate from KEY_PEOPLE_CONTACTS.md in the project repo, which tracks advisors and leads already in motion (Tarpy, Delaney, Wake County Beekeepers, Julia Mahood, etc.). Once outreach starts here, it's worth mirroring status updates into that file too so both stay in sync.</t>
+          <t>Batches so far: Core advisors (3, added Jul 25 2026) — Seeley, Tarpy, Delaney. Batch 1 (19, Jul 25 2026) — national spread. Batch 2 (6, Jul 25 2026) — Southeast-focused (Clemson, UT Knoxville, LSU, WVU, Appalachian State, UF Extension). 28 contacts total.</t>
         </is>
       </c>
     </row>
@@ -2077,7 +2248,17 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>All contacts are faculty PIs / program directors / lead specialists — no grad students or postdocs included in either batch, per your instruction to keep this to PI-level contacts.</t>
+          <t>This list is separate from KEY_PEOPLE_CONTACTS.md in the project repo, which tracks advisors and leads already in motion. Once outreach starts here, it's worth mirroring status updates into that file too so both stay in sync.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>All contacts are faculty PIs / program directors / lead specialists — no grad students or postdocs included, per your instruction to keep this to PI-level contacts.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Julia Mahood to contacts tracker, mark as contacted
</commit_message>
<xml_diff>
--- a/University_Bee_Research_Contacts.xlsx
+++ b/University_Bee_Research_Contacts.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'University Contacts'!$A$1:$L$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'University Contacts'!$A$1:$L$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -616,8 +616,8 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J2" s="9" t="inlineStr"/>
-      <c r="K2" s="9" t="inlineStr"/>
+      <c r="J2" s="9" t="n"/>
+      <c r="K2" s="9" t="n"/>
       <c r="L2" s="9" t="inlineStr">
         <is>
           <t>Extremely high-value contact - worth a personally written email referencing the 2015 Apidologie paper rather than the generic boilerplate.</t>
@@ -650,7 +650,7 @@
           <t>drtarpy@ncsu.edu</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr"/>
+      <c r="F3" s="9" t="n"/>
       <c r="G3" s="9" t="inlineStr">
         <is>
           <t>Behavioral ecology of honey bee queens (polyandry, intracolony genetic diversity), social immunity, IPM, queen reproductive quality</t>
@@ -666,8 +666,8 @@
           <t>Confirmed - Advisor</t>
         </is>
       </c>
-      <c r="J3" s="9" t="inlineStr"/>
-      <c r="K3" s="9" t="inlineStr"/>
+      <c r="J3" s="9" t="n"/>
+      <c r="K3" s="9" t="n"/>
       <c r="L3" s="9" t="inlineStr">
         <is>
           <t>Already actively engaged - not part of the cold-outreach batches below. Included here so this list reads as complete when shared with him. See MEETING_NOTES_2026-07-21_Tarpy.md for full context.</t>
@@ -725,102 +725,106 @@
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="K4" s="9" t="inlineStr"/>
+      <c r="K4" s="9" t="n"/>
       <c r="L4" s="9" t="inlineStr">
         <is>
           <t>Reintroduction email sent 2026-07-25 (see delaney-email.html / KEY_PEOPLE_CONTACTS.md). Not part of the cold-outreach batches below - included here so this list reads as complete when shared with Tarpy.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="60" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Dr. Christina Grozinger</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Professor of Entomology; Director, Center for Pollinator Research</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Penn State University</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Atlantic</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>cmgrozinger@psu.edu</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>814-865-2214</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Molecular/physiological/ecological determinants of managed &amp; wild bee health; pollinator conservation</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Directs one of the largest pollinator research centers in the US, with a strong extension/outreach arm that could amplify a citizen-science mapping project.</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Not Contacted</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="n"/>
-      <c r="K5" s="2" t="n"/>
-      <c r="L5" s="2" t="n"/>
+    <row r="5" ht="70" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Julia Mahood</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Georgia Master Craft Beekeeper; Founder, Map My DCA</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Independent (Map My DCA / Metro Atlanta Beekeepers Association / Georgia Beekeepers Association)</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Southeast</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>info@mapmydca.com (also admin@mapmydca.com)</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr"/>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>Citizen-science mapping of honey bee drone congregation areas (DCAs) using UAV-mounted queen pheromone lures</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>Very close citizen-science cousin to SaveTheHives - the app already has a 'DCA Mapping' feature marked 'coming soon.' 2018 Georgia Beekeeper of the Year; guest on Beekeeping Today and OSU Extension's PolliNation podcasts.</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>Emailed - Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="inlineStr"/>
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>Sent via mapmydca.com/contact-us/ (no personal email published) - date is approximate/session date, correct if off. See KEY_PEOPLE_CONTACTS.md.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Dr. Marla Spivak</t>
+          <t>Dr. Christina Grozinger</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Professor Emeritus (MacArthur Fellow); Bee Lab</t>
+          <t>Professor of Entomology; Director, Center for Pollinator Research</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>University of Minnesota</t>
+          <t>Penn State University</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>Mid-Atlantic</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Use beelab.umn.edu/contact form</t>
+          <t>cmgrozinger@psu.edu</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>612-624-3636 (dept.)</t>
+          <t>814-865-2214</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Honey bee social immunity, hygienic behavior, breeding for disease resistance</t>
+          <t>Molecular/physiological/ecological determinants of managed &amp; wild bee health; pollinator conservation</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>The 'Genetic Goldmine' framing (survivor colonies bred for resistance) is essentially her life's work; a major name if she engages, even briefly.</t>
+          <t>Directs one of the largest pollinator research centers in the US, with a strong extension/outreach arm that could amplify a citizen-science mapping project.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -830,51 +834,47 @@
       </c>
       <c r="J6" s="2" t="n"/>
       <c r="K6" s="2" t="n"/>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>Emeritus - personal email not published; route through lab contact form or department (entomology@umn.edu).</t>
-        </is>
-      </c>
+      <c r="L6" s="2" t="n"/>
     </row>
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Dr. Elina Nino</t>
+          <t>Dr. Marla Spivak</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Professor of Cooperative Extension, Apiculture</t>
+          <t>Professor Emeritus (MacArthur Fellow); Bee Lab</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>UC Davis (Harry H. Laidlaw Jr. Honey Bee Research Facility)</t>
+          <t>University of Minnesota</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>West/Pacific</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>elnino@ucdavis.edu</t>
+          <t>Use beelab.umn.edu/contact form</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>(530) 752-1011</t>
+          <t>612-624-3636 (dept.)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Queen health, colony management, statewide extension</t>
+          <t>Honey bee social immunity, hygienic behavior, breeding for disease resistance</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>West Coast counterpart to NC State's program; UC Davis runs one of the country's top honey bee research facilities.</t>
+          <t>The 'Genetic Goldmine' framing (survivor colonies bred for resistance) is essentially her life's work; a major name if she engages, even briefly.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -884,47 +884,51 @@
       </c>
       <c r="J7" s="2" t="n"/>
       <c r="K7" s="2" t="n"/>
-      <c r="L7" s="2" t="n"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Emeritus - personal email not published; route through lab contact form or department (entomology@umn.edu).</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="60" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Dr. Juliana Rangel</t>
+          <t>Dr. Elina Nino</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Associate Professor of Apiculture</t>
+          <t>Professor of Cooperative Extension, Apiculture</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Texas A&amp;M University</t>
+          <t>UC Davis (Harry H. Laidlaw Jr. Honey Bee Research Facility)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>South Central</t>
+          <t>West/Pacific</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>juliana.rangelposada@ag.tamu.edu</t>
+          <t>elnino@ucdavis.edu</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>979-845-1074</t>
+          <t>(530) 752-1011</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Queen and drone reproductive biology, colony health</t>
+          <t>Queen health, colony management, statewide extension</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Leads a major state bee program in a region with a strong feral/Africanized colony research thread already in our contact notes.</t>
+          <t>West Coast counterpart to NC State's program; UC Davis runs one of the country's top honey bee research facilities.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -939,42 +943,42 @@
     <row r="9" ht="60" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Dr. Jamie Ellis</t>
+          <t>Dr. Juliana Rangel</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Gahan Endowed Professor; Director, Honey Bee Research &amp; Extension Lab</t>
+          <t>Associate Professor of Apiculture</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>University of Florida</t>
+          <t>Texas A&amp;M University</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>South Central</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>jdellis@ufl.edu</t>
+          <t>juliana.rangelposada@ag.tamu.edu</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>352-273-3924</t>
+          <t>979-845-1074</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Colony health, feral colony/swarm removal and trapping, extension</t>
+          <t>Queen and drone reproductive biology, colony health</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>HBREL runs active feral-colony removal and trapping research - closely adjacent to SaveTheHives' core mapping mission.</t>
+          <t>Leads a major state bee program in a region with a strong feral/Africanized colony research thread already in our contact notes.</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -989,38 +993,42 @@
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Dr. Brandon Hopkins</t>
+          <t>Dr. Jamie Ellis</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Thurber Endowed Distinguished Professor of Pollinator Ecology</t>
+          <t>Gahan Endowed Professor; Director, Honey Bee Research &amp; Extension Lab</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Washington State University</t>
+          <t>University of Florida</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Pacific Northwest</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>bhopkins@wsu.edu</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="n"/>
+          <t>jdellis@ufl.edu</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>352-273-3924</t>
+        </is>
+      </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Honey bee germplasm cryopreservation, genetic diversity preservation</t>
+          <t>Colony health, feral colony/swarm removal and trapping, extension</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Genetic-diversity/germplasm preservation work lines up directly with the 'Genetic Goldmine' survivor-genetics framing.</t>
+          <t>HBREL runs active feral-colony removal and trapping research - closely adjacent to SaveTheHives' core mapping mission.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1030,51 +1038,43 @@
       </c>
       <c r="J10" s="2" t="n"/>
       <c r="K10" s="2" t="n"/>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>Succeeded Steve Sheppard (retired 2024) as program lead.</t>
-        </is>
-      </c>
+      <c r="L10" s="2" t="n"/>
     </row>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Dr. Reed Johnson</t>
+          <t>Dr. Brandon Hopkins</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Associate Professor, Bee Lab</t>
+          <t>Thurber Endowed Distinguished Professor of Pollinator Ecology</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Ohio State University</t>
+          <t>Washington State University</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>Pacific Northwest</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>johnson.5005@osu.edu</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>(330) 202-3523</t>
-        </is>
-      </c>
+          <t>bhopkins@wsu.edu</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Foraging ecology, pesticide exposure</t>
+          <t>Honey bee germplasm cryopreservation, genetic diversity preservation</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Strong Midwest program with an active beekeeper-facing extension arm.</t>
+          <t>Genetic-diversity/germplasm preservation work lines up directly with the 'Genetic Goldmine' survivor-genetics framing.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1084,43 +1084,51 @@
       </c>
       <c r="J11" s="2" t="n"/>
       <c r="K11" s="2" t="n"/>
-      <c r="L11" s="2" t="n"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Succeeded Steve Sheppard (retired 2024) as program lead.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Dr. Scott McArt</t>
+          <t>Dr. Reed Johnson</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Associate Professor of Pollinator Health; Director, Dyce Lab for Honey Bee Studies</t>
+          <t>Associate Professor, Bee Lab</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Cornell University</t>
+          <t>Ohio State University</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Northeast</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>shm33@cornell.edu</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="n"/>
+          <t>johnson.5005@osu.edu</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>(330) 202-3523</t>
+        </is>
+      </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Pesticide and pathogen impacts on pollinator health</t>
+          <t>Foraging ecology, pesticide exposure</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Northeast counterpart to Tarpy's NC State program; Dyce Lab has a large beekeeper-facing extension program to cross-promote with.</t>
+          <t>Strong Midwest program with an active beekeeper-facing extension arm.</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1130,51 +1138,43 @@
       </c>
       <c r="J12" s="2" t="n"/>
       <c r="K12" s="2" t="n"/>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>General lab inbox is dycelab@cornell.edu if personal email bounces.</t>
-        </is>
-      </c>
+      <c r="L12" s="2" t="n"/>
     </row>
     <row r="13" ht="60" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Dr. Keith Delaplane</t>
+          <t>Dr. Scott McArt</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Professor Emeritus; Director, UGA Bee Program</t>
+          <t>Associate Professor of Pollinator Health; Director, Dyce Lab for Honey Bee Studies</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>University of Georgia</t>
+          <t>Cornell University</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Northeast</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>ksd@uga.edu</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>706-542-2816</t>
-        </is>
-      </c>
+          <t>shm33@cornell.edu</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n"/>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Colony health, honey bee biology and behavior, IPM</t>
+          <t>Pesticide and pathogen impacts on pollinator health</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Adjacent Southeast state; UGA runs a large Master Beekeeper Program that could help cross-promote SaveTheHives.</t>
+          <t>Northeast counterpart to Tarpy's NC State program; Dyce Lab has a large beekeeper-facing extension program to cross-promote with.</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1184,22 +1184,26 @@
       </c>
       <c r="J13" s="2" t="n"/>
       <c r="K13" s="2" t="n"/>
-      <c r="L13" s="2" t="n"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>General lab inbox is dycelab@cornell.edu if personal email bounces.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="60" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Dr. Geoff Williams</t>
+          <t>Dr. Keith Delaplane</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Associate Professor; Director, Bee Center</t>
+          <t>Professor Emeritus; Director, UGA Bee Program</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Auburn University</t>
+          <t>University of Georgia</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1209,22 +1213,22 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>williams@auburn.edu</t>
+          <t>ksd@uga.edu</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>(334) 844-5068</t>
+          <t>706-542-2816</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Colony health, disease and stressor interactions</t>
+          <t>Colony health, honey bee biology and behavior, IPM</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Adjacent Southeast state with a growing, well-funded bee center.</t>
+          <t>Adjacent Southeast state; UGA runs a large Master Beekeeper Program that could help cross-promote SaveTheHives.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1239,42 +1243,42 @@
     <row r="15" ht="60" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Dr. Ramesh Sagili</t>
+          <t>Dr. Geoff Williams</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Professor of Apiculture, Honey Bee Lab</t>
+          <t>Associate Professor; Director, Bee Center</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Oregon State University</t>
+          <t>Auburn University</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Pacific Northwest</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>ramesh.sagili@oregonstate.edu</t>
+          <t>williams@auburn.edu</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>541-737-5460</t>
+          <t>(334) 844-5068</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Nutrition, Varroa management, pollination</t>
+          <t>Colony health, disease and stressor interactions</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>West Coast program with an active Master Beekeeper Program and strong grower/beekeeper outreach.</t>
+          <t>Adjacent Southeast state with a growing, well-funded bee center.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1284,51 +1288,47 @@
       </c>
       <c r="J15" s="2" t="n"/>
       <c r="K15" s="2" t="n"/>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>Email inferred from standard OSU firstname.lastname pattern - confirm before sending (site lists it as an obfuscated mailto).</t>
-        </is>
-      </c>
+      <c r="L15" s="2" t="n"/>
     </row>
     <row r="16" ht="60" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Dr. Dennis vanEngelsdorp</t>
+          <t>Dr. Ramesh Sagili</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Professor; Chief Scientist, Bee Informed Partnership</t>
+          <t>Professor of Apiculture, Honey Bee Lab</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>University of Maryland</t>
+          <t>Oregon State University</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Mid-Atlantic</t>
+          <t>Pacific Northwest</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>dvane@umd.edu</t>
+          <t>ramesh.sagili@oregonstate.edu</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>301-405-3911</t>
+          <t>541-737-5460</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Epidemiological approach to colony loss; large-scale citizen-science monitoring</t>
+          <t>Nutrition, Varroa management, pollination</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Runs the country's largest citizen-science bee health survey (the annual national Colony Loss Survey) - the closest methodological cousin to SaveTheHives on this list.</t>
+          <t>West Coast program with an active Master Beekeeper Program and strong grower/beekeeper outreach.</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1340,49 +1340,49 @@
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Strong candidate to lead with - his own work is citizen-science-adjacent.</t>
+          <t>Email inferred from standard OSU firstname.lastname pattern - confirm before sending (site lists it as an obfuscated mailto).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="60" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Krispn Given</t>
+          <t>Dr. Dennis vanEngelsdorp</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Senior Apiculture Specialist, Honey Bee Breeding Program</t>
+          <t>Professor; Chief Scientist, Bee Informed Partnership</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Purdue University</t>
+          <t>University of Maryland</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>Mid-Atlantic</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>kgiven@purdue.edu</t>
+          <t>dvane@umd.edu</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>765-494-6747</t>
+          <t>301-405-3911</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Mite-resistant honey bee breeding</t>
+          <t>Epidemiological approach to colony loss; large-scale citizen-science monitoring</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Directly on-thesis: breeding survivor stock for Varroa resistance.</t>
+          <t>Runs the country's largest citizen-science bee health survey (the annual national Colony Loss Survey) - the closest methodological cousin to SaveTheHives on this list.</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1392,22 +1392,26 @@
       </c>
       <c r="J17" s="2" t="n"/>
       <c r="K17" s="2" t="n"/>
-      <c r="L17" s="2" t="n"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Strong candidate to lead with - his own work is citizen-science-adjacent.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="60" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Dr. Meghan Milbrath</t>
+          <t>Krispn Given</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Academic Specialist; Coordinator, Michigan Pollinator Initiative</t>
+          <t>Senior Apiculture Specialist, Honey Bee Breeding Program</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Michigan State University</t>
+          <t>Purdue University</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1417,22 +1421,22 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>honeybees@msu.edu</t>
+          <t>kgiven@purdue.edu</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>(517) 884-9518</t>
+          <t>765-494-6747</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Bacterial pathogens, honey bee medicine, risk assessment</t>
+          <t>Mite-resistant honey bee breeding</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Trains veterinary students/professionals in honey bee medicine - an outreach channel beyond the typical beekeeping audience.</t>
+          <t>Directly on-thesis: breeding survivor stock for Varroa resistance.</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1442,51 +1446,47 @@
       </c>
       <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="n"/>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>Lab inbox shown; address email to Dr. Milbrath by name.</t>
-        </is>
-      </c>
+      <c r="L18" s="2" t="n"/>
     </row>
     <row r="19" ht="60" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Dr. Jeff Harris</t>
+          <t>Dr. Meghan Milbrath</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Associate Professor, Apiculture Extension Specialist</t>
+          <t>Academic Specialist; Coordinator, Michigan Pollinator Initiative</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Mississippi State University</t>
+          <t>Michigan State University</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>jeff.harris@msstate.edu</t>
+          <t>honeybees@msu.edu</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>662-325-2085</t>
+          <t>(517) 884-9518</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Varroa-resistant stock breeding, colony health</t>
+          <t>Bacterial pathogens, honey bee medicine, risk assessment</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Deep South program with a breeding focus that aligns closely with the Genetic Goldmine framing.</t>
+          <t>Trains veterinary students/professionals in honey bee medicine - an outreach channel beyond the typical beekeeping audience.</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -1496,47 +1496,51 @@
       </c>
       <c r="J19" s="2" t="n"/>
       <c r="K19" s="2" t="n"/>
-      <c r="L19" s="2" t="n"/>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Lab inbox shown; address email to Dr. Milbrath by name.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="60" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Dr. Adam Dolezal</t>
+          <t>Dr. Jeff Harris</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Associate Professor, Dolezal Bee Research Lab</t>
+          <t>Associate Professor, Apiculture Extension Specialist</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>University of Illinois Urbana-Champaign</t>
+          <t>Mississippi State University</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>adolezal@illinois.edu</t>
+          <t>jeff.harris@msstate.edu</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>217-300-6762</t>
+          <t>662-325-2085</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Colony nutrition/stress, virus transmission between managed and wild bees</t>
+          <t>Varroa-resistant stock breeding, colony health</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Studies wild-managed bee interactions directly relevant to feral colony tracking.</t>
+          <t>Deep South program with a breeding focus that aligns closely with the Genetic Goldmine framing.</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -1551,42 +1555,42 @@
     <row r="21" ht="60" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Dr. Neelendra Joshi</t>
+          <t>Dr. Adam Dolezal</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Professor, Apiculture &amp; Pollinator Health</t>
+          <t>Associate Professor, Dolezal Bee Research Lab</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>University of Arkansas</t>
+          <t>University of Illinois Urbana-Champaign</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>South Central</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>nkjoshi@uark.edu</t>
+          <t>adolezal@illinois.edu</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>(479) 575-3872</t>
+          <t>217-300-6762</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Toxicology, pollinator ecology and health</t>
+          <t>Colony nutrition/stress, virus transmission between managed and wild bees</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Fills a south-central US research gap in this list.</t>
+          <t>Studies wild-managed bee interactions directly relevant to feral colony tracking.</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -1601,42 +1605,42 @@
     <row r="22" ht="60" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Dr. Judy Wu-Smart</t>
+          <t>Dr. Neelendra Joshi</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Associate Professor, Bee Lab</t>
+          <t>Professor, Apiculture &amp; Pollinator Health</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>University of Nebraska-Lincoln</t>
+          <t>University of Arkansas</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Great Plains</t>
+          <t>South Central</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>jwu-smart@unl.edu</t>
+          <t>nkjoshi@uark.edu</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>402-472-8696</t>
+          <t>(479) 575-3872</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Pollinator health, pesticide exposure</t>
+          <t>Toxicology, pollinator ecology and health</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Great Plains program; trained under Marla Spivak, a nice connective thread if both are contacted.</t>
+          <t>Fills a south-central US research gap in this list.</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1651,38 +1655,42 @@
     <row r="23" ht="60" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Dr. Margaret Couvillon</t>
+          <t>Dr. Judy Wu-Smart</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Associate Professor, Pollinator Biology and Ecology</t>
+          <t>Associate Professor, Bee Lab</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Virginia Tech</t>
+          <t>University of Nebraska-Lincoln</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Mid-Atlantic</t>
+          <t>Great Plains</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>mjc@vt.edu</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="n"/>
+          <t>jwu-smart@unl.edu</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>402-472-8696</t>
+        </is>
+      </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Honey bee foraging, recruitment, waggle-dance communication</t>
+          <t>Pollinator health, pesticide exposure</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Adjacent to NC/VA; foraging-ecology research could make direct use of SaveTheHives' colony location data.</t>
+          <t>Great Plains program; trained under Marla Spivak, a nice connective thread if both are contacted.</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -1697,42 +1705,38 @@
     <row r="24" ht="60" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Ben Powell</t>
+          <t>Dr. Margaret Couvillon</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Coordinator, Apiculture and Pollinator Program</t>
+          <t>Associate Professor, Pollinator Biology and Ecology</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Clemson University</t>
+          <t>Virginia Tech</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Mid-Atlantic</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>bpowel2@clemson.edu</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>843-662-3526</t>
-        </is>
-      </c>
+          <t>mjc@vt.edu</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Extension support for SC beekeepers, pollinator conservation outreach</t>
+          <t>Honey bee foraging, recruitment, waggle-dance communication</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Neighboring state extension program (SC) with an active beekeeper-facing newsletter (CAPPings) that could carry a SaveTheHives mention statewide.</t>
+          <t>Adjacent to NC/VA; foraging-ecology research could make direct use of SaveTheHives' colony location data.</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1747,17 +1751,17 @@
     <row r="25" ht="60" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Dr. Jennifer Tsuruda</t>
+          <t>Ben Powell</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor; Apiculture Extension Specialist</t>
+          <t>Coordinator, Apiculture and Pollinator Program</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>University of Tennessee, Knoxville</t>
+          <t>Clemson University</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1767,18 +1771,22 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>jennifer.tsuruda@utk.edu</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="n"/>
+          <t>bpowel2@clemson.edu</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>843-662-3526</t>
+        </is>
+      </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Honey bee health and management, pollination, beekeeper education</t>
+          <t>Extension support for SC beekeepers, pollinator conservation outreach</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Runs the TN Master Beekeeping Program (previously at Clemson) - a large existing beekeeper network one door down from NC.</t>
+          <t>Neighboring state extension program (SC) with an active beekeeper-facing newsletter (CAPPings) that could carry a SaveTheHives mention statewide.</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -1788,26 +1796,22 @@
       </c>
       <c r="J25" s="2" t="n"/>
       <c r="K25" s="2" t="n"/>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>Email inferred from standard UTK firstname.lastname pattern - confirm before sending.</t>
-        </is>
-      </c>
+      <c r="L25" s="2" t="n"/>
     </row>
     <row r="26" ht="60" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Dr. Morgan Christman</t>
+          <t>Dr. Jennifer Tsuruda</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor of Pollinator Ecology</t>
+          <t>Assistant Professor; Apiculture Extension Specialist</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>LSU AgCenter / Louisiana State University</t>
+          <t>University of Tennessee, Knoxville</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1817,18 +1821,18 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>MChristman@agcenter.lsu.edu</t>
+          <t>jennifer.tsuruda@utk.edu</t>
         </is>
       </c>
       <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Pollinator ecology and conservation; building baseline pollinator/native bee data for Louisiana</t>
+          <t>Honey bee health and management, pollination, beekeeper education</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Brand-new program (2025) actively building citizen-science partnerships (a Louisiana Bumble Bee Atlas) - likely receptive to a sister citizen-science project.</t>
+          <t>Runs the TN Master Beekeeping Program (previously at Clemson) - a large existing beekeeper network one door down from NC.</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -1838,47 +1842,47 @@
       </c>
       <c r="J26" s="2" t="n"/>
       <c r="K26" s="2" t="n"/>
-      <c r="L26" s="2" t="n"/>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Email inferred from standard UTK firstname.lastname pattern - confirm before sending.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="60" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Dr. Yong-Lak Park</t>
+          <t>Dr. Morgan Christman</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Professor of Entomology</t>
+          <t>Assistant Professor of Pollinator Ecology</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>West Virginia University</t>
+          <t>LSU AgCenter / Louisiana State University</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Mid-Atlantic</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Yong-Lak.Park@mail.wvu.edu</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>(304) 293-2882</t>
-        </is>
-      </c>
+          <t>MChristman@agcenter.lsu.edu</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Integrated pest management, pollination ecology of solitary/wild bees, geospatial/remote-sensing methods</t>
+          <t>Pollinator ecology and conservation; building baseline pollinator/native bee data for Louisiana</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>His geospatial/remote-sensing angle on wild bee ecology is a natural methodological conversation with a location-mapping app.</t>
+          <t>Brand-new program (2025) actively building citizen-science partnerships (a Louisiana Bumble Bee Atlas) - likely receptive to a sister citizen-science project.</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -1888,51 +1892,47 @@
       </c>
       <c r="J27" s="2" t="n"/>
       <c r="K27" s="2" t="n"/>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>Focus is broader than honey bees specifically (solitary bees, IPM) - tailor the relevance line accordingly.</t>
-        </is>
-      </c>
+      <c r="L27" s="2" t="n"/>
     </row>
     <row r="28" ht="60" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Dr. Rahman Tashakkori</t>
+          <t>Dr. Yong-Lak Park</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Lowe's Distinguished Professor of Computer Science; PI, AppMAIS Project</t>
+          <t>Professor of Entomology</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Appalachian State University</t>
+          <t>West Virginia University</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Mid-Atlantic</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>tashakkorir@appstate.edu</t>
+          <t>Yong-Lak.Park@mail.wvu.edu</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>(828) 262-7009</t>
+          <t>(304) 293-2882</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Honey bee health monitoring systems (hive sensors, data science, AI) - the AppMAIS/Beemon project</t>
+          <t>Integrated pest management, pollination ecology of solitary/wild bees, geospatial/remote-sensing methods</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Closest technical cousin on this whole list: an NC-based (Boone) honeybee data/monitoring project. Strong potential collaborator, not just an outreach target - worth a more tailored note than the standard boilerplate.</t>
+          <t>His geospatial/remote-sensing angle on wild bee ecology is a natural methodological conversation with a location-mapping app.</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -1944,24 +1944,24 @@
       <c r="K28" s="2" t="n"/>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>Computer Science, not entomology/biology - AppMAIS is the hook, not a traditional bee lab.</t>
+          <t>Focus is broader than honey bees specifically (solitary bees, IPM) - tailor the relevance line accordingly.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="60" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Amy Vu</t>
+          <t>Dr. Rahman Tashakkori</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>State Specialized Extension Agent II, Apiculture</t>
+          <t>Lowe's Distinguished Professor of Computer Science; PI, AppMAIS Project</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>University of Florida (Honey Bee Research &amp; Extension Lab)</t>
+          <t>Appalachian State University</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1971,18 +1971,22 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>amy.vu@ufl.edu</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="n"/>
+          <t>tashakkorir@appstate.edu</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>(828) 262-7009</t>
+        </is>
+      </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Beekeeper education, UF Master Beekeeper Program, Bee College, extension outreach</t>
+          <t>Honey bee health monitoring systems (hive sensors, data science, AI) - the AppMAIS/Beemon project</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Runs UF's beekeeper-facing extension/outreach programs (Bee College, Master Beekeeper Program) - a second, extension-focused UF contact alongside Dr. Ellis's research-focused one.</t>
+          <t>Closest technical cousin on this whole list: an NC-based (Boone) honeybee data/monitoring project. Strong potential collaborator, not just an outreach target - worth a more tailored note than the standard boilerplate.</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -1994,17 +1998,67 @@
       <c r="K29" s="2" t="n"/>
       <c r="L29" s="2" t="inlineStr">
         <is>
+          <t>Computer Science, not entomology/biology - AppMAIS is the hook, not a traditional bee lab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="60" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Amy Vu</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>State Specialized Extension Agent II, Apiculture</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>University of Florida (Honey Bee Research &amp; Extension Lab)</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Southeast</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>amy.vu@ufl.edu</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Beekeeper education, UF Master Beekeeper Program, Bee College, extension outreach</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Runs UF's beekeeper-facing extension/outreach programs (Bee College, Master Beekeeper Program) - a second, extension-focused UF contact alongside Dr. Ellis's research-focused one.</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="n"/>
+      <c r="K30" s="2" t="n"/>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
           <t>Same institution as Jamie Ellis (already on this list) but a distinct extension-facing role - fine to contact both.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L29"/>
+  <autoFilter ref="A1:L30"/>
   <dataValidations count="2">
-    <dataValidation sqref="I2:I29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Contacted,Emailed - Awaiting Reply,Replied,Call/Meeting Scheduled,Declined,No Longer Pursuing,Confirmed - Advisor"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Northeast,Mid-Atlantic,Southeast,Midwest,Great Plains,South Central,Mountain West,Pacific Northwest,West/Pacific"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2173,7 +2227,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Purpose: track outreach to university honey bee / apiculture research programs that may want to know about savethehives.org.</t>
+          <t>Purpose: track outreach to university honey bee / apiculture research programs (plus a few key independent contacts) that may want to know about savethehives.org.</t>
         </is>
       </c>
     </row>
@@ -2183,7 +2237,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Rows 2-4 (highlighted): Dr. Thomas Seeley (Cornell), Dr. David Tarpy (NC State), and Dr. Debbie Delaney (U Delaware) — the three researchers already central to this project. Tarpy is a confirmed named advisor; Delaney was emailed 2026-07-25 and is awaiting reply; Seeley is the scientific originator of the wild-colony-survival research this project's framing is built on, and has co-authored with the other two. They're listed first, separately from the batches below, so the sheet reads as complete at a glance if shared with Tarpy.</t>
+          <t>Rows 2-5 (highlighted): Dr. Thomas Seeley (Cornell), Dr. David Tarpy (NC State), Dr. Debbie Delaney (U Delaware), and Julia Mahood (Map My DCA, Atlanta) — contacts already central to or already in motion for this project, listed first and separately from the batches below so the sheet reads as complete at a glance if shared with Tarpy. Tarpy is a confirmed named advisor; Delaney and Mahood were emailed 2026-07-25 and are awaiting reply; Seeley is not yet contacted but is the scientific originator of the wild-colony-survival research this project's framing is built on.</t>
         </is>
       </c>
     </row>
@@ -2238,7 +2292,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Batches so far: Core advisors (3, added Jul 25 2026) — Seeley, Tarpy, Delaney. Batch 1 (19, Jul 25 2026) — national spread. Batch 2 (6, Jul 25 2026) — Southeast-focused (Clemson, UT Knoxville, LSU, WVU, Appalachian State, UF Extension). 28 contacts total.</t>
+          <t>Batches so far: Already-in-motion contacts (4, added Jul 25 2026) — Seeley, Tarpy, Delaney, Mahood. Batch 1 (19, Jul 25 2026) — national spread. Batch 2 (6, Jul 25 2026) — Southeast-focused (Clemson, UT Knoxville, LSU, WVU, Appalachian State, UF Extension). 29 contacts total.</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2312,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>All contacts are faculty PIs / program directors / lead specialists — no grad students or postdocs included, per your instruction to keep this to PI-level contacts.</t>
+          <t>Most contacts are university faculty PIs / program directors / lead specialists (no grad students or postdocs, per your instruction). Julia Mahood is the one non-university exception, included because she's already an active lead/contact for this project.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add planned send date tracking with color-coded scheduling
</commit_message>
<xml_diff>
--- a/University_Bee_Research_Contacts.xlsx
+++ b/University_Bee_Research_Contacts.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'University Contacts'!$A$1:$L$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'University Contacts'!$A$1:$M$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="7">
     <font>
       <name val="Calibri"/>
@@ -105,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -126,10 +128,42 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F8CBCB"/>
+          <bgColor rgb="00F8CBCB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C9EAD3"/>
+          <bgColor rgb="00C9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00CFE2F3"/>
+          <bgColor rgb="00CFE2F3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -491,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:M30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -503,9 +537,10 @@
     <col width="34" customWidth="1" min="7" max="7"/>
     <col width="40" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -556,15 +591,20 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Planned Send Date</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Date Emailed</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Follow-up Date</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -616,9 +656,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J2" s="9" t="n"/>
+      <c r="J2" s="10" t="n">
+        <v>46232</v>
+      </c>
       <c r="K2" s="9" t="n"/>
-      <c r="L2" s="9" t="inlineStr">
+      <c r="L2" s="9" t="n"/>
+      <c r="M2" s="9" t="inlineStr">
         <is>
           <t>Extremely high-value contact - worth a personally written email referencing the 2015 Apidologie paper rather than the generic boilerplate.</t>
         </is>
@@ -668,7 +711,8 @@
       </c>
       <c r="J3" s="9" t="n"/>
       <c r="K3" s="9" t="n"/>
-      <c r="L3" s="9" t="inlineStr">
+      <c r="L3" s="9" t="n"/>
+      <c r="M3" s="9" t="inlineStr">
         <is>
           <t>Already actively engaged - not part of the cold-outreach batches below. Included here so this list reads as complete when shared with him. See MEETING_NOTES_2026-07-21_Tarpy.md for full context.</t>
         </is>
@@ -720,13 +764,14 @@
           <t>Emailed - Awaiting Reply</t>
         </is>
       </c>
-      <c r="J4" s="9" t="inlineStr">
+      <c r="J4" s="9" t="n"/>
+      <c r="K4" s="9" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="K4" s="9" t="n"/>
-      <c r="L4" s="9" t="inlineStr">
+      <c r="L4" s="9" t="n"/>
+      <c r="M4" s="9" t="inlineStr">
         <is>
           <t>Reintroduction email sent 2026-07-25 (see delaney-email.html / KEY_PEOPLE_CONTACTS.md). Not part of the cold-outreach batches below - included here so this list reads as complete when shared with Tarpy.</t>
         </is>
@@ -758,7 +803,7 @@
           <t>info@mapmydca.com (also admin@mapmydca.com)</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr"/>
+      <c r="F5" s="9" t="n"/>
       <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Citizen-science mapping of honey bee drone congregation areas (DCAs) using UAV-mounted queen pheromone lures</t>
@@ -774,13 +819,14 @@
           <t>Emailed - Awaiting Reply</t>
         </is>
       </c>
-      <c r="J5" s="9" t="inlineStr">
+      <c r="J5" s="9" t="n"/>
+      <c r="K5" s="9" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="K5" s="9" t="inlineStr"/>
-      <c r="L5" s="9" t="inlineStr">
+      <c r="L5" s="9" t="n"/>
+      <c r="M5" s="9" t="inlineStr">
         <is>
           <t>Sent via mapmydca.com/contact-us/ (no personal email published) - date is approximate/session date, correct if off. See KEY_PEOPLE_CONTACTS.md.</t>
         </is>
@@ -832,9 +878,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J6" s="2" t="n"/>
+      <c r="J6" s="11" t="n">
+        <v>46239</v>
+      </c>
       <c r="K6" s="2" t="n"/>
       <c r="L6" s="2" t="n"/>
+      <c r="M6" s="2" t="n"/>
     </row>
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -882,9 +931,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J7" s="2" t="n"/>
+      <c r="J7" s="11" t="n">
+        <v>46273</v>
+      </c>
       <c r="K7" s="2" t="n"/>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="n"/>
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Emeritus - personal email not published; route through lab contact form or department (entomology@umn.edu).</t>
         </is>
@@ -936,9 +988,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J8" s="2" t="n"/>
+      <c r="J8" s="11" t="n">
+        <v>46273</v>
+      </c>
       <c r="K8" s="2" t="n"/>
       <c r="L8" s="2" t="n"/>
+      <c r="M8" s="2" t="n"/>
     </row>
     <row r="9" ht="60" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -986,9 +1041,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J9" s="2" t="n"/>
+      <c r="J9" s="11" t="n">
+        <v>46273</v>
+      </c>
       <c r="K9" s="2" t="n"/>
       <c r="L9" s="2" t="n"/>
+      <c r="M9" s="2" t="n"/>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -1036,9 +1094,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J10" s="2" t="n"/>
+      <c r="J10" s="11" t="n">
+        <v>46274</v>
+      </c>
       <c r="K10" s="2" t="n"/>
       <c r="L10" s="2" t="n"/>
+      <c r="M10" s="2" t="n"/>
     </row>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -1082,9 +1143,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J11" s="2" t="n"/>
+      <c r="J11" s="11" t="n">
+        <v>46274</v>
+      </c>
       <c r="K11" s="2" t="n"/>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="n"/>
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>Succeeded Steve Sheppard (retired 2024) as program lead.</t>
         </is>
@@ -1136,9 +1200,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J12" s="2" t="n"/>
+      <c r="J12" s="11" t="n">
+        <v>46274</v>
+      </c>
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="n"/>
+      <c r="M12" s="2" t="n"/>
     </row>
     <row r="13" ht="60" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
@@ -1182,9 +1249,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J13" s="2" t="n"/>
+      <c r="J13" s="11" t="n">
+        <v>46275</v>
+      </c>
       <c r="K13" s="2" t="n"/>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="n"/>
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>General lab inbox is dycelab@cornell.edu if personal email bounces.</t>
         </is>
@@ -1236,9 +1306,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J14" s="2" t="n"/>
+      <c r="J14" s="11" t="n">
+        <v>46275</v>
+      </c>
       <c r="K14" s="2" t="n"/>
       <c r="L14" s="2" t="n"/>
+      <c r="M14" s="2" t="n"/>
     </row>
     <row r="15" ht="60" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -1286,9 +1359,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J15" s="2" t="n"/>
+      <c r="J15" s="11" t="n">
+        <v>46275</v>
+      </c>
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="n"/>
+      <c r="M15" s="2" t="n"/>
     </row>
     <row r="16" ht="60" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -1336,9 +1412,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J16" s="2" t="n"/>
+      <c r="J16" s="11" t="n">
+        <v>46280</v>
+      </c>
       <c r="K16" s="2" t="n"/>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="n"/>
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>Email inferred from standard OSU firstname.lastname pattern - confirm before sending (site lists it as an obfuscated mailto).</t>
         </is>
@@ -1390,9 +1469,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J17" s="2" t="n"/>
+      <c r="J17" s="11" t="n">
+        <v>46238</v>
+      </c>
       <c r="K17" s="2" t="n"/>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="n"/>
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>Strong candidate to lead with - his own work is citizen-science-adjacent.</t>
         </is>
@@ -1444,9 +1526,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J18" s="2" t="n"/>
+      <c r="J18" s="11" t="n">
+        <v>46280</v>
+      </c>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="n"/>
+      <c r="M18" s="2" t="n"/>
     </row>
     <row r="19" ht="60" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
@@ -1494,9 +1579,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J19" s="2" t="n"/>
+      <c r="J19" s="11" t="n">
+        <v>46280</v>
+      </c>
       <c r="K19" s="2" t="n"/>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="n"/>
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>Lab inbox shown; address email to Dr. Milbrath by name.</t>
         </is>
@@ -1548,9 +1636,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J20" s="2" t="n"/>
+      <c r="J20" s="11" t="n">
+        <v>46281</v>
+      </c>
       <c r="K20" s="2" t="n"/>
       <c r="L20" s="2" t="n"/>
+      <c r="M20" s="2" t="n"/>
     </row>
     <row r="21" ht="60" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
@@ -1598,9 +1689,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J21" s="2" t="n"/>
+      <c r="J21" s="11" t="n">
+        <v>46240</v>
+      </c>
       <c r="K21" s="2" t="n"/>
       <c r="L21" s="2" t="n"/>
+      <c r="M21" s="2" t="n"/>
     </row>
     <row r="22" ht="60" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -1648,9 +1742,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J22" s="2" t="n"/>
+      <c r="J22" s="11" t="n">
+        <v>46281</v>
+      </c>
       <c r="K22" s="2" t="n"/>
       <c r="L22" s="2" t="n"/>
+      <c r="M22" s="2" t="n"/>
     </row>
     <row r="23" ht="60" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
@@ -1698,9 +1795,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J23" s="2" t="n"/>
+      <c r="J23" s="11" t="n">
+        <v>46281</v>
+      </c>
       <c r="K23" s="2" t="n"/>
       <c r="L23" s="2" t="n"/>
+      <c r="M23" s="2" t="n"/>
     </row>
     <row r="24" ht="60" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -1744,9 +1844,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J24" s="2" t="n"/>
+      <c r="J24" s="11" t="n">
+        <v>46282</v>
+      </c>
       <c r="K24" s="2" t="n"/>
       <c r="L24" s="2" t="n"/>
+      <c r="M24" s="2" t="n"/>
     </row>
     <row r="25" ht="60" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
@@ -1794,9 +1897,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J25" s="2" t="n"/>
+      <c r="J25" s="11" t="n">
+        <v>46282</v>
+      </c>
       <c r="K25" s="2" t="n"/>
       <c r="L25" s="2" t="n"/>
+      <c r="M25" s="2" t="n"/>
     </row>
     <row r="26" ht="60" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -1840,9 +1946,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J26" s="2" t="n"/>
+      <c r="J26" s="11" t="n">
+        <v>46282</v>
+      </c>
       <c r="K26" s="2" t="n"/>
-      <c r="L26" s="2" t="inlineStr">
+      <c r="L26" s="2" t="n"/>
+      <c r="M26" s="2" t="inlineStr">
         <is>
           <t>Email inferred from standard UTK firstname.lastname pattern - confirm before sending.</t>
         </is>
@@ -1890,9 +1999,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J27" s="2" t="n"/>
+      <c r="J27" s="11" t="n">
+        <v>46231</v>
+      </c>
       <c r="K27" s="2" t="n"/>
       <c r="L27" s="2" t="n"/>
+      <c r="M27" s="2" t="n"/>
     </row>
     <row r="28" ht="60" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
@@ -1940,9 +2052,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J28" s="2" t="n"/>
+      <c r="J28" s="11" t="n">
+        <v>46287</v>
+      </c>
       <c r="K28" s="2" t="n"/>
-      <c r="L28" s="2" t="inlineStr">
+      <c r="L28" s="2" t="n"/>
+      <c r="M28" s="2" t="inlineStr">
         <is>
           <t>Focus is broader than honey bees specifically (solitary bees, IPM) - tailor the relevance line accordingly.</t>
         </is>
@@ -1994,9 +2109,12 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J29" s="2" t="n"/>
+      <c r="J29" s="11" t="n">
+        <v>46233</v>
+      </c>
       <c r="K29" s="2" t="n"/>
-      <c r="L29" s="2" t="inlineStr">
+      <c r="L29" s="2" t="n"/>
+      <c r="M29" s="2" t="inlineStr">
         <is>
           <t>Computer Science, not entomology/biology - AppMAIS is the hook, not a traditional bee lab.</t>
         </is>
@@ -2044,16 +2162,30 @@
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J30" s="2" t="n"/>
+      <c r="J30" s="11" t="n">
+        <v>46287</v>
+      </c>
       <c r="K30" s="2" t="n"/>
-      <c r="L30" s="2" t="inlineStr">
+      <c r="L30" s="2" t="n"/>
+      <c r="M30" s="2" t="inlineStr">
         <is>
           <t>Same institution as Jamie Ellis (already on this list) but a distinct extension-facing role - fine to contact both.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L30"/>
+  <autoFilter ref="A1:M30"/>
+  <conditionalFormatting sqref="J2:J30">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>AND(J2&lt;&gt;"",J2&lt;=TODAY())</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>AND(J2&lt;&gt;"",J2&gt;TODAY(),J2&lt;=TODAY()+14)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2">
+      <formula>J2&gt;TODAY()+14</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation sqref="I2:I30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Contacted,Emailed - Awaiting Reply,Replied,Call/Meeting Scheduled,Declined,No Longer Pursuing,Confirmed - Advisor"</formula1>
@@ -2208,10 +2340,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="115" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2237,7 +2369,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Rows 2-5 (highlighted): Dr. Thomas Seeley (Cornell), Dr. David Tarpy (NC State), Dr. Debbie Delaney (U Delaware), and Julia Mahood (Map My DCA, Atlanta) — contacts already central to or already in motion for this project, listed first and separately from the batches below so the sheet reads as complete at a glance if shared with Tarpy. Tarpy is a confirmed named advisor; Delaney and Mahood were emailed 2026-07-25 and are awaiting reply; Seeley is not yet contacted but is the scientific originator of the wild-colony-survival research this project's framing is built on.</t>
+          <t>Rows 2-5 (highlighted tan): Dr. Thomas Seeley (Cornell), Dr. David Tarpy (NC State), Dr. Debbie Delaney (U Delaware), and Julia Mahood (Map My DCA, Atlanta) — contacts already central to or already in motion for this project, listed first so the sheet reads as complete at a glance if shared with Tarpy.</t>
         </is>
       </c>
     </row>
@@ -2247,42 +2379,42 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>How to use this sheet:</t>
+          <t>Column J, Planned Send Date, and what the colors mean:</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>1. Update the Status dropdown (column I) as you email each contact: Not Contacted -&gt; Emailed - Awaiting Reply -&gt; Replied / Call-Meeting Scheduled / Declined / No Longer Pursuing / Confirmed - Advisor.</t>
+          <t>- Blank: already actioned (Tarpy/Delaney/Mahood) or no date set yet.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>2. Fill in Date Emailed (column J) when you send the first email.</t>
+          <t>- Red/pink: due or overdue — the planned date has arrived or passed and it hasn't been sent.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>3. Set a Follow-up Date (column K) — a reasonable rule of thumb is 2-3 weeks after the initial email if there's been no reply.</t>
+          <t>- Green: coming up in the next 14 days — a near-term reminder to draft and send.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>4. Use Notes (column L) for anything short and specific: what they said, a call summary, a second contact they mentioned, etc.</t>
+          <t>- Blue: scheduled further out — no action needed yet.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>5. US Region (column D) is a dropdown too, in case you add more contacts later and want the categories to stay consistent: Northeast, Mid-Atlantic, Southeast, Midwest, Great Plains, South Central, Mountain West, Pacific Northwest, West/Pacific.</t>
+          <t>These colors update automatically based on today's date each time you open the file.</t>
         </is>
       </c>
     </row>
@@ -2292,7 +2424,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Batches so far: Already-in-motion contacts (4, added Jul 25 2026) — Seeley, Tarpy, Delaney, Mahood. Batch 1 (19, Jul 25 2026) — national spread. Batch 2 (6, Jul 25 2026) — Southeast-focused (Clemson, UT Knoxville, LSU, WVU, Appalachian State, UF Extension). 29 contacts total.</t>
+          <t>Why the dates are staggered the way they are: 6 contacts are scheduled soon (late Jul - early Aug 2026) because they're less tied to the summer beekeeping field-day calendar — an emeritus researcher (Seeley), a computer-science PI (Tashakkori) whose teaching load is lighter over summer, a brand-new hire actively building partnerships (Christman), a center director (Grozinger), a lab-based researcher (Dolezal), and a data-survey specialist whose busy season is fall/winter (vanEngelsdorp). The other 20 — mostly extension apiculturists running summer field days and Master Beekeeper programs — are staggered after Labor Day (Sept 8, 2026 onward), 3 per day on Tuesdays/Wednesdays/Thursdays, to avoid a mass-blast pattern and land in inboxes when they're actually checking email regularly.</t>
         </is>
       </c>
     </row>
@@ -2302,17 +2434,69 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>This list is separate from KEY_PEOPLE_CONTACTS.md in the project repo, which tracks advisors and leads already in motion. Once outreach starts here, it's worth mirroring status updates into that file too so both stay in sync.</t>
+          <t>How to use this sheet:</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr"/>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>1. Update the Status dropdown (column I) as you email each contact: Not Contacted -&gt; Emailed - Awaiting Reply -&gt; Replied / Call-Meeting Scheduled / Declined / No Longer Pursuing / Confirmed - Advisor.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Most contacts are university faculty PIs / program directors / lead specialists (no grad students or postdocs, per your instruction). Julia Mahood is the one non-university exception, included because she's already an active lead/contact for this project.</t>
+          <t>2. Adjust Planned Send Date (column J) any time — drag rows around, push dates out, whatever fits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>3. Fill in Date Emailed (column K) when you actually send.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>4. Set a Follow-up Date (column L) — 2-3 weeks after sending is a reasonable default if there's no reply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>5. Use Notes (column M) for anything short and specific.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>6. US Region (column D) is a dropdown too, in case you add more contacts later and want the categories to stay consistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Batches so far: Already-in-motion (4, Jul 25 2026) — Seeley, Tarpy, Delaney, Mahood. Batch 1 (19, Jul 25 2026) — national spread. Batch 2 (6, Jul 25 2026) — Southeast-focused. 29 contacts total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>This list is separate from KEY_PEOPLE_CONTACTS.md in the project repo. Once outreach starts, it's worth mirroring status updates into that file too so both stay in sync.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add department links and SAS Institute connection column
</commit_message>
<xml_diff>
--- a/University_Bee_Research_Contacts.xlsx
+++ b/University_Bee_Research_Contacts.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'University Contacts'!$A$1:$M$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'University Contacts'!$A$1:$O$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,10 +20,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,8 +61,14 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -78,6 +85,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFF3D6"/>
         <bgColor rgb="00FFF3D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+        <bgColor rgb="00D9EAD3"/>
       </patternFill>
     </fill>
   </fills>
@@ -107,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -132,6 +145,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -525,22 +553,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M30"/>
+  <dimension ref="A1:O30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="34" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -561,56 +591,66 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Department / Lab Link</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>US Region</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Research Focus</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Why Relevant to SaveTheHives</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>SAS Software Connection</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Planned Send Date</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Date Emailed</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Follow-up Date</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="70" customHeight="1">
+    <row r="2" ht="90" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
           <t>Dr. Thomas D. Seeley</t>
@@ -626,48 +666,58 @@
           <t>Cornell University</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>https://as.cornell.edu/people/thomas-seeley</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
         <is>
           <t>Northeast</t>
         </is>
       </c>
-      <c r="E2" s="9" t="inlineStr">
+      <c r="F2" s="9" t="inlineStr">
         <is>
           <t>tds5@cornell.edu</t>
         </is>
       </c>
-      <c r="F2" s="9" t="inlineStr">
+      <c r="G2" s="9" t="inlineStr">
         <is>
           <t>(607) 279-5498</t>
         </is>
       </c>
-      <c r="G2" s="9" t="inlineStr">
+      <c r="H2" s="9" t="inlineStr">
         <is>
           <t>Swarm intelligence and collective decision-making in honey bee colonies; wild/feral colony survival without Varroa treatment (Arnot Forest, NY, ongoing since 2011)</t>
         </is>
       </c>
-      <c r="H2" s="9" t="inlineStr">
+      <c r="I2" s="9" t="inlineStr">
         <is>
           <t>The scientific foundation of the whole 'Genetic Goldmine' framing: his Arnot Forest feral-colony study is the original long-running demonstration that untreated wild colonies persist and adapt to Varroa. Author of Honeybee Democracy and The Lives of Bees. Already a co-author with Tarpy and Delaney (Seeley, Tarpy, Griffin, Carcione, Delaney 2015, Apidologie) on wild colony genetic structure - arguably the single most on-thesis name on this whole list.</t>
         </is>
       </c>
-      <c r="I2" s="9" t="inlineStr">
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>Confirmed — Cornell IT holds a campus-wide SAS site license (Base/SAS, SAS/STAT, Enterprise Guide, etc.) available to faculty, staff, and students.</t>
+        </is>
+      </c>
+      <c r="K2" s="9" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J2" s="10" t="n">
+      <c r="L2" s="12" t="n">
         <v>46232</v>
       </c>
-      <c r="K2" s="9" t="n"/>
-      <c r="L2" s="9" t="n"/>
-      <c r="M2" s="9" t="inlineStr">
+      <c r="M2" s="9" t="n"/>
+      <c r="N2" s="9" t="n"/>
+      <c r="O2" s="9" t="inlineStr">
         <is>
           <t>Extremely high-value contact - worth a personally written email referencing the 2015 Apidologie paper rather than the generic boilerplate.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="70" customHeight="1">
+    <row r="3" ht="90" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Dr. David R. Tarpy</t>
@@ -683,42 +733,52 @@
           <t>NC State University</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
+        <is>
+          <t>https://ncsuapiculture.net/</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>Southeast</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>drtarpy@ncsu.edu</t>
         </is>
       </c>
-      <c r="F3" s="9" t="n"/>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="G3" s="9" t="n"/>
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>Behavioral ecology of honey bee queens (polyandry, intracolony genetic diversity), social immunity, IPM, queen reproductive quality</t>
         </is>
       </c>
-      <c r="H3" s="9" t="inlineStr">
+      <c r="I3" s="9" t="inlineStr">
         <is>
           <t>Named scientific advisor on SaveTheHives' 'Genetic Goldmine' framing since the Jul 21 2026 lunch meeting - reviewed and approved all 5 questions on the language handout. Helped get the original savethehives.com press coverage in 2008.</t>
         </is>
       </c>
-      <c r="I3" s="9" t="inlineStr">
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>Exceptional — SAS Institute was literally founded at NC State (1966) as an agricultural-data research project - Jim Goodnight and colleagues built the original SAS there before spinning it out in 1976. SAS Hall (math/stats building) is named for the founders, and SAS still actively partners with NC State's Plant Sciences Initiative. Hard to beat as a personal connection.</t>
+        </is>
+      </c>
+      <c r="K3" s="9" t="inlineStr">
         <is>
           <t>Confirmed - Advisor</t>
         </is>
       </c>
-      <c r="J3" s="9" t="n"/>
-      <c r="K3" s="9" t="n"/>
       <c r="L3" s="9" t="n"/>
-      <c r="M3" s="9" t="inlineStr">
+      <c r="M3" s="9" t="n"/>
+      <c r="N3" s="9" t="n"/>
+      <c r="O3" s="9" t="inlineStr">
         <is>
           <t>Already actively engaged - not part of the cold-outreach batches below. Included here so this list reads as complete when shared with him. See MEETING_NOTES_2026-07-21_Tarpy.md for full context.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="70" customHeight="1">
+    <row r="4" ht="90" customHeight="1">
       <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Dr. Debbie Delaney</t>
@@ -734,50 +794,60 @@
           <t>University of Delaware</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>https://www.udel.edu/canr/departments/entomology-and-wildlife-ecology/faculty-staff/debbie-delaney/</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>Mid-Atlantic</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>dadelane@udel.edu</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="G4" s="9" t="inlineStr">
         <is>
           <t>302-831-8883</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="H4" s="9" t="inlineStr">
         <is>
           <t>Evolutionary biology and population genetics of honey bees, benefits of polyandry on colony health, IPM</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="I4" s="9" t="inlineStr">
         <is>
           <t>Her UD faculty page lists savethehives.com as one of her own resource links - she was directly involved with the original 2008-era project alongside Tarpy. Co-author with Tarpy and Seeley on the 2015 Apidologie survivor-colony genetics paper - directly on-thesis for the Genetic Goldmine framing.</t>
         </is>
       </c>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>Confirmed — UD licenses SAS for teaching and research (annual license via UDeploy), sub-licensable by departments.</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
         <is>
           <t>Emailed - Awaiting Reply</t>
-        </is>
-      </c>
-      <c r="J4" s="9" t="n"/>
-      <c r="K4" s="9" t="inlineStr">
-        <is>
-          <t>2026-07-25</t>
         </is>
       </c>
       <c r="L4" s="9" t="n"/>
       <c r="M4" s="9" t="inlineStr">
         <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="N4" s="9" t="n"/>
+      <c r="O4" s="9" t="inlineStr">
+        <is>
           <t>Reintroduction email sent 2026-07-25 (see delaney-email.html / KEY_PEOPLE_CONTACTS.md). Not part of the cold-outreach batches below - included here so this list reads as complete when shared with Tarpy.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="70" customHeight="1">
+    <row r="5" ht="90" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Julia Mahood</t>
@@ -793,46 +863,56 @@
           <t>Independent (Map My DCA / Metro Atlanta Beekeepers Association / Georgia Beekeepers Association)</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>https://mapmydca.com/about-us/</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>Southeast</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>info@mapmydca.com (also admin@mapmydca.com)</t>
         </is>
       </c>
-      <c r="F5" s="9" t="n"/>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="G5" s="9" t="n"/>
+      <c r="H5" s="9" t="inlineStr">
         <is>
           <t>Citizen-science mapping of honey bee drone congregation areas (DCAs) using UAV-mounted queen pheromone lures</t>
         </is>
       </c>
-      <c r="H5" s="9" t="inlineStr">
+      <c r="I5" s="9" t="inlineStr">
         <is>
           <t>Very close citizen-science cousin to SaveTheHives - the app already has a 'DCA Mapping' feature marked 'coming soon.' 2018 Georgia Beekeeper of the Year; guest on Beekeeping Today and OSU Extension's PolliNation podcasts.</t>
         </is>
       </c>
-      <c r="I5" s="9" t="inlineStr">
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>Not researched</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="inlineStr">
         <is>
           <t>Emailed - Awaiting Reply</t>
-        </is>
-      </c>
-      <c r="J5" s="9" t="n"/>
-      <c r="K5" s="9" t="inlineStr">
-        <is>
-          <t>2026-07-25</t>
         </is>
       </c>
       <c r="L5" s="9" t="n"/>
       <c r="M5" s="9" t="inlineStr">
         <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="N5" s="9" t="n"/>
+      <c r="O5" s="9" t="inlineStr">
+        <is>
           <t>Sent via mapmydca.com/contact-us/ (no personal email published) - date is approximate/session date, correct if off. See KEY_PEOPLE_CONTACTS.md.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1">
+    <row r="6" ht="80" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Dr. Christina Grozinger</t>
@@ -848,44 +928,54 @@
           <t>Penn State University</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>https://pollinators.psu.edu/about/directory/christina-grozinger-ph-d</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Mid-Atlantic</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>cmgrozinger@psu.edu</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>814-865-2214</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Molecular/physiological/ecological determinants of managed &amp; wild bee health; pollinator conservation</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Directs one of the largest pollinator research centers in the US, with a strong extension/outreach arm that could amplify a citizen-science mapping project.</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed — Penn State distributes SAS 9.4 licenses to faculty/staff/students through its Software Store, renewed annually.</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J6" s="11" t="n">
+      <c r="L6" s="14" t="n">
         <v>46239</v>
       </c>
-      <c r="K6" s="2" t="n"/>
-      <c r="L6" s="2" t="n"/>
       <c r="M6" s="2" t="n"/>
-    </row>
-    <row r="7" ht="60" customHeight="1">
+      <c r="N6" s="2" t="n"/>
+      <c r="O6" s="2" t="n"/>
+    </row>
+    <row r="7" ht="80" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Dr. Marla Spivak</t>
@@ -901,48 +991,58 @@
           <t>University of Minnesota</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>https://entomology.umn.edu/people/marla-spivak</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Midwest</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Use beelab.umn.edu/contact form</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>612-624-3636 (dept.)</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Honey bee social immunity, hygienic behavior, breeding for disease resistance</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>The 'Genetic Goldmine' framing (survivor colonies bred for resistance) is essentially her life's work; a major name if she engages, even briefly.</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed — SAS is licensed campus-wide through IT@UMN for teaching, learning, and research.</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J7" s="11" t="n">
+      <c r="L7" s="14" t="n">
         <v>46273</v>
       </c>
-      <c r="K7" s="2" t="n"/>
-      <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M7" s="2" t="n"/>
+      <c r="N7" s="2" t="n"/>
+      <c r="O7" s="2" t="inlineStr">
         <is>
           <t>Emeritus - personal email not published; route through lab contact form or department (entomology@umn.edu).</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1">
+    <row r="8" ht="80" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Dr. Elina Nino</t>
@@ -958,44 +1058,54 @@
           <t>UC Davis (Harry H. Laidlaw Jr. Honey Bee Research Facility)</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>https://elninobeelab.ucdavis.edu/people/elina-nino</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>West/Pacific</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>elnino@ucdavis.edu</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>(530) 752-1011</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Queen health, colony management, statewide extension</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>West Coast counterpart to NC State's program; UC Davis runs one of the country's top honey bee research facilities.</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Not confirmed — UC Davis's Computational Research Service prominently licenses SPSS; no clear public SAS-specific site license page turned up in search. Worth asking Dr. Niño directly rather than assuming.</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J8" s="11" t="n">
+      <c r="L8" s="14" t="n">
         <v>46273</v>
       </c>
-      <c r="K8" s="2" t="n"/>
-      <c r="L8" s="2" t="n"/>
       <c r="M8" s="2" t="n"/>
-    </row>
-    <row r="9" ht="60" customHeight="1">
+      <c r="N8" s="2" t="n"/>
+      <c r="O8" s="2" t="n"/>
+    </row>
+    <row r="9" ht="80" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Dr. Juliana Rangel</t>
@@ -1011,44 +1121,54 @@
           <t>Texas A&amp;M University</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>https://honeybeelab.tamu.edu</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>South Central</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>juliana.rangelposada@ag.tamu.edu</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>979-845-1074</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Queen and drone reproductive biology, colony health</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Leads a major state bee program in a region with a strong feral/Africanized colony research thread already in our contact notes.</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed — SAS is available through the Texas A&amp;M Software Center and is used directly in the Statistics department's curriculum.</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J9" s="11" t="n">
+      <c r="L9" s="14" t="n">
         <v>46273</v>
       </c>
-      <c r="K9" s="2" t="n"/>
-      <c r="L9" s="2" t="n"/>
       <c r="M9" s="2" t="n"/>
-    </row>
-    <row r="10" ht="60" customHeight="1">
+      <c r="N9" s="2" t="n"/>
+      <c r="O9" s="2" t="n"/>
+    </row>
+    <row r="10" ht="80" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Dr. Jamie Ellis</t>
@@ -1064,44 +1184,54 @@
           <t>University of Florida</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>https://entnemdept.ufl.edu/honey-bee/about-us/people/jamie-ellis/</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Southeast</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>jdellis@ufl.edu</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>352-273-3924</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Colony health, feral colony/swarm removal and trapping, extension</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>HBREL runs active feral-colony removal and trapping research - closely adjacent to SaveTheHives' core mapping mission.</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed — UF provides free SAS 9.4 access via remote desktop, plus discounted student installs.</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J10" s="11" t="n">
+      <c r="L10" s="14" t="n">
         <v>46274</v>
       </c>
-      <c r="K10" s="2" t="n"/>
-      <c r="L10" s="2" t="n"/>
       <c r="M10" s="2" t="n"/>
-    </row>
-    <row r="11" ht="60" customHeight="1">
+      <c r="N10" s="2" t="n"/>
+      <c r="O10" s="2" t="n"/>
+    </row>
+    <row r="11" ht="80" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Dr. Brandon Hopkins</t>
@@ -1117,44 +1247,54 @@
           <t>Washington State University</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>https://labs.wsu.edu/hopkinslab/</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>Pacific Northwest</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>bhopkins@wsu.edu</t>
         </is>
       </c>
-      <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Honey bee germplasm cryopreservation, genetic diversity preservation</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Genetic-diversity/germplasm preservation work lines up directly with the 'Genetic Goldmine' survivor-genetics framing.</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed — SAS is available via WSU's Software Site License, with CAHNRS (the ag college) specifically licensing it for Biological Systems Engineering.</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J11" s="11" t="n">
+      <c r="L11" s="14" t="n">
         <v>46274</v>
       </c>
-      <c r="K11" s="2" t="n"/>
-      <c r="L11" s="2" t="n"/>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M11" s="2" t="n"/>
+      <c r="N11" s="2" t="n"/>
+      <c r="O11" s="2" t="inlineStr">
         <is>
           <t>Succeeded Steve Sheppard (retired 2024) as program lead.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="60" customHeight="1">
+    <row r="12" ht="80" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Dr. Reed Johnson</t>
@@ -1170,44 +1310,54 @@
           <t>Ohio State University</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>https://entomology.osu.edu/our-people/reed-johnson</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>Midwest</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>johnson.5005@osu.edu</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>(330) 202-3523</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Foraging ecology, pesticide exposure</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Strong Midwest program with an active beekeeper-facing extension arm.</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed — Ohio State licenses both Teaching/Research and Administrative versions of SAS campus-wide, renewed each September; the Statistics department actively supports it.</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J12" s="11" t="n">
+      <c r="L12" s="14" t="n">
         <v>46274</v>
       </c>
-      <c r="K12" s="2" t="n"/>
-      <c r="L12" s="2" t="n"/>
       <c r="M12" s="2" t="n"/>
-    </row>
-    <row r="13" ht="60" customHeight="1">
+      <c r="N12" s="2" t="n"/>
+      <c r="O12" s="2" t="n"/>
+    </row>
+    <row r="13" ht="80" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Dr. Scott McArt</t>
@@ -1223,44 +1373,54 @@
           <t>Cornell University</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>https://blogs.cornell.edu/dycelab/</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>Northeast</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>shm33@cornell.edu</t>
         </is>
       </c>
-      <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Pesticide and pathogen impacts on pollinator health</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Northeast counterpart to Tarpy's NC State program; Dyce Lab has a large beekeeper-facing extension program to cross-promote with.</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed — Cornell IT holds a campus-wide SAS site license (Base/SAS, SAS/STAT, Enterprise Guide, etc.) available to faculty, staff, and students.</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J13" s="11" t="n">
+      <c r="L13" s="14" t="n">
         <v>46275</v>
       </c>
-      <c r="K13" s="2" t="n"/>
-      <c r="L13" s="2" t="n"/>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M13" s="2" t="n"/>
+      <c r="N13" s="2" t="n"/>
+      <c r="O13" s="2" t="inlineStr">
         <is>
           <t>General lab inbox is dycelab@cornell.edu if personal email bounces.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1">
+    <row r="14" ht="80" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Dr. Keith Delaplane</t>
@@ -1276,44 +1436,54 @@
           <t>University of Georgia</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>https://ent.uga.edu/people/faculty/keith-delaplane.html</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Southeast</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>ksd@uga.edu</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>706-542-2816</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Colony health, honey bee biology and behavior, IPM</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>Adjacent Southeast state; UGA runs a large Master Beekeeper Program that could help cross-promote SaveTheHives.</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Not confirmed — Found SAS access via special Data Services workstations in the library, but no clear campus-wide site license page. Worth asking Delaplane directly rather than assuming.</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J14" s="11" t="n">
+      <c r="L14" s="14" t="n">
         <v>46275</v>
       </c>
-      <c r="K14" s="2" t="n"/>
-      <c r="L14" s="2" t="n"/>
       <c r="M14" s="2" t="n"/>
-    </row>
-    <row r="15" ht="60" customHeight="1">
+      <c r="N14" s="2" t="n"/>
+      <c r="O14" s="2" t="n"/>
+    </row>
+    <row r="15" ht="80" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Dr. Geoff Williams</t>
@@ -1329,44 +1499,54 @@
           <t>Auburn University</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>https://agriculture.auburn.edu/enpp/bee-center/team.php</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>Southeast</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>williams@auburn.edu</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>(334) 844-5068</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Colony health, disease and stressor interactions</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>Adjacent Southeast state with a growing, well-funded bee center.</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed — Auburn's College of Agriculture runs a dedicated 'SAS and R Statistical Software Resources' page - directly relevant since Williams is in that college.</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J15" s="11" t="n">
+      <c r="L15" s="14" t="n">
         <v>46275</v>
       </c>
-      <c r="K15" s="2" t="n"/>
-      <c r="L15" s="2" t="n"/>
       <c r="M15" s="2" t="n"/>
-    </row>
-    <row r="16" ht="60" customHeight="1">
+      <c r="N15" s="2" t="n"/>
+      <c r="O15" s="2" t="n"/>
+    </row>
+    <row r="16" ht="80" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Dr. Ramesh Sagili</t>
@@ -1382,48 +1562,58 @@
           <t>Oregon State University</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>https://honeybeelab.oregonstate.edu/users/ramesh-sagili</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Pacific Northwest</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>ramesh.sagili@oregonstate.edu</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>541-737-5460</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Nutrition, Varroa management, pollination</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>West Coast program with an active Master Beekeeper Program and strong grower/beekeeper outreach.</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed — OSU participates in a campus-wide SAS site license; College of Forestry has its own block of 75 licenses.</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J16" s="11" t="n">
+      <c r="L16" s="14" t="n">
         <v>46280</v>
       </c>
-      <c r="K16" s="2" t="n"/>
-      <c r="L16" s="2" t="n"/>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="M16" s="2" t="n"/>
+      <c r="N16" s="2" t="n"/>
+      <c r="O16" s="2" t="inlineStr">
         <is>
           <t>Email inferred from standard OSU firstname.lastname pattern - confirm before sending (site lists it as an obfuscated mailto).</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="60" customHeight="1">
+    <row r="17" ht="80" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Dr. Dennis vanEngelsdorp</t>
@@ -1439,48 +1629,58 @@
           <t>University of Maryland</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>https://entomology.umd.edu/people/dennis-vanengelsdorp</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>Mid-Atlantic</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>dvane@umd.edu</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>301-405-3911</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Epidemiological approach to colony loss; large-scale citizen-science monitoring</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>Runs the country's largest citizen-science bee health survey (the annual national Colony Loss Survey) - the closest methodological cousin to SaveTheHives on this list.</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed — UMD DivIT sells and renews SAS licenses for teaching/research use.</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J17" s="11" t="n">
+      <c r="L17" s="14" t="n">
         <v>46238</v>
       </c>
-      <c r="K17" s="2" t="n"/>
-      <c r="L17" s="2" t="n"/>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="M17" s="2" t="n"/>
+      <c r="N17" s="2" t="n"/>
+      <c r="O17" s="2" t="inlineStr">
         <is>
           <t>Strong candidate to lead with - his own work is citizen-science-adjacent.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="60" customHeight="1">
+    <row r="18" ht="80" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Krispn Given</t>
@@ -1496,44 +1696,54 @@
           <t>Purdue University</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D18" s="16" t="inlineStr">
+        <is>
+          <t>https://extension.entm.purdue.edu/beehive/</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>Midwest</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>kgiven@purdue.edu</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>765-494-6747</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Mite-resistant honey bee breeding</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>Directly on-thesis: breeding survivor stock for Varroa resistance.</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed — SAS is available through Purdue's Research Computing (RCAC) and supported by the Statistics department's free consulting service.</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J18" s="11" t="n">
+      <c r="L18" s="14" t="n">
         <v>46280</v>
       </c>
-      <c r="K18" s="2" t="n"/>
-      <c r="L18" s="2" t="n"/>
       <c r="M18" s="2" t="n"/>
-    </row>
-    <row r="19" ht="60" customHeight="1">
+      <c r="N18" s="2" t="n"/>
+      <c r="O18" s="2" t="n"/>
+    </row>
+    <row r="19" ht="80" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Dr. Meghan Milbrath</t>
@@ -1549,48 +1759,58 @@
           <t>Michigan State University</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>https://milbrathlab.msu.edu/</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>Midwest</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>honeybees@msu.edu</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>(517) 884-9518</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>Bacterial pathogens, honey bee medicine, risk assessment</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>Trains veterinary students/professionals in honey bee medicine - an outreach channel beyond the typical beekeeping audience.</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Not confirmed — Search kept surfacing University of Michigan instead of MSU; no clear MSU-specific SAS site license page found. Worth asking Milbrath directly rather than assuming.</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J19" s="11" t="n">
+      <c r="L19" s="14" t="n">
         <v>46280</v>
       </c>
-      <c r="K19" s="2" t="n"/>
-      <c r="L19" s="2" t="n"/>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="M19" s="2" t="n"/>
+      <c r="N19" s="2" t="n"/>
+      <c r="O19" s="2" t="inlineStr">
         <is>
           <t>Lab inbox shown; address email to Dr. Milbrath by name.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1">
+    <row r="20" ht="80" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Dr. Jeff Harris</t>
@@ -1606,44 +1826,54 @@
           <t>Mississippi State University</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>https://extension.msstate.edu/directory/dr-jeffrey-harris</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>Southeast</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>jeff.harris@msstate.edu</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>662-325-2085</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>Varroa-resistant stock breeding, colony health</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>Deep South program with a breeding focus that aligns closely with the Genetic Goldmine framing.</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed — MSU holds a limited campus site license for SAS, with public access via the Mitchell Memorial Library Computer Commons.</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J20" s="11" t="n">
+      <c r="L20" s="14" t="n">
         <v>46281</v>
       </c>
-      <c r="K20" s="2" t="n"/>
-      <c r="L20" s="2" t="n"/>
       <c r="M20" s="2" t="n"/>
-    </row>
-    <row r="21" ht="60" customHeight="1">
+      <c r="N20" s="2" t="n"/>
+      <c r="O20" s="2" t="n"/>
+    </row>
+    <row r="21" ht="80" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Dr. Adam Dolezal</t>
@@ -1659,44 +1889,54 @@
           <t>University of Illinois Urbana-Champaign</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>https://publish.illinois.edu/dolezalbeelab/</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Midwest</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>adolezal@illinois.edu</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>217-300-6762</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>Colony nutrition/stress, virus transmission between managed and wild bees</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>Studies wild-managed bee interactions directly relevant to feral colony tracking.</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed — SAS Education Analytical Suite is distributed campus-wide via the Illinois WebStore.</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J21" s="11" t="n">
+      <c r="L21" s="14" t="n">
         <v>46240</v>
       </c>
-      <c r="K21" s="2" t="n"/>
-      <c r="L21" s="2" t="n"/>
       <c r="M21" s="2" t="n"/>
-    </row>
-    <row r="22" ht="60" customHeight="1">
+      <c r="N21" s="2" t="n"/>
+      <c r="O21" s="2" t="n"/>
+    </row>
+    <row r="22" ht="80" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Dr. Neelendra Joshi</t>
@@ -1712,44 +1952,54 @@
           <t>University of Arkansas</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>https://enpl.uark.edu/people/faculty/uid/nkjoshi/name/Neelendra+Joshi/</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>South Central</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>nkjoshi@uark.edu</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>(479) 575-3872</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>Toxicology, pollinator ecology and health</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>Fills a south-central US research gap in this list.</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed — SAS site licenses are free for faculty and students, distributed via sitelicense.uark.edu.</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J22" s="11" t="n">
+      <c r="L22" s="14" t="n">
         <v>46281</v>
       </c>
-      <c r="K22" s="2" t="n"/>
-      <c r="L22" s="2" t="n"/>
       <c r="M22" s="2" t="n"/>
-    </row>
-    <row r="23" ht="60" customHeight="1">
+      <c r="N22" s="2" t="n"/>
+      <c r="O22" s="2" t="n"/>
+    </row>
+    <row r="23" ht="80" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Dr. Judy Wu-Smart</t>
@@ -1765,44 +2015,54 @@
           <t>University of Nebraska-Lincoln</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>https://entomology.unl.edu/person/dr-judy-wu-smart/</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>Great Plains</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>jwu-smart@unl.edu</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>402-472-8696</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>Pollinator health, pesticide exposure</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>Great Plains program; trained under Marla Spivak, a nice connective thread if both are contacted.</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed — UNL struck a new no-cost enterprise-wide SAS agreement in Oct 2024, and hosts an active local Nebraska SAS Users Group (NEBSUG) for training/networking.</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J23" s="11" t="n">
+      <c r="L23" s="14" t="n">
         <v>46281</v>
       </c>
-      <c r="K23" s="2" t="n"/>
-      <c r="L23" s="2" t="n"/>
       <c r="M23" s="2" t="n"/>
-    </row>
-    <row r="24" ht="60" customHeight="1">
+      <c r="N23" s="2" t="n"/>
+      <c r="O23" s="2" t="n"/>
+    </row>
+    <row r="24" ht="80" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Dr. Margaret Couvillon</t>
@@ -1818,40 +2078,50 @@
           <t>Virginia Tech</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>https://www.ento.vt.edu/people/Faculty0/Couvillon.html</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>Mid-Atlantic</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>mjc@vt.edu</t>
         </is>
       </c>
-      <c r="F24" s="2" t="n"/>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Honey bee foraging, recruitment, waggle-dance communication</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>Adjacent to NC/VA; foraging-ecology research could make direct use of SaveTheHives' colony location data.</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed — SAS is available via VT Software Distribution, and VT's Statistical Applications and Innovation Group (SAIG) supports it directly.</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J24" s="11" t="n">
+      <c r="L24" s="14" t="n">
         <v>46282</v>
       </c>
-      <c r="K24" s="2" t="n"/>
-      <c r="L24" s="2" t="n"/>
       <c r="M24" s="2" t="n"/>
-    </row>
-    <row r="25" ht="60" customHeight="1">
+      <c r="N24" s="2" t="n"/>
+      <c r="O24" s="2" t="n"/>
+    </row>
+    <row r="25" ht="80" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
           <t>Ben Powell</t>
@@ -1867,44 +2137,54 @@
           <t>Clemson University</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>https://www.clemson.edu/extension/apiculture-pollinators/</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>Southeast</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>bpowel2@clemson.edu</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>843-662-3526</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>Extension support for SC beekeepers, pollinator conservation outreach</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>Neighboring state extension program (SC) with an active beekeeper-facing newsletter (CAPPings) that could carry a SaveTheHives mention statewide.</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="J25" s="13" t="inlineStr">
+        <is>
+          <t>Exceptional — SAS gifted Clemson $3.3M in software licensing (2021, renewed through 2026) covering Base SAS and cloud-based SAS Viya for ~25,000 users, specifically to power big-data/analytics research and teaching.</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J25" s="11" t="n">
+      <c r="L25" s="14" t="n">
         <v>46282</v>
       </c>
-      <c r="K25" s="2" t="n"/>
-      <c r="L25" s="2" t="n"/>
       <c r="M25" s="2" t="n"/>
-    </row>
-    <row r="26" ht="60" customHeight="1">
+      <c r="N25" s="2" t="n"/>
+      <c r="O25" s="2" t="n"/>
+    </row>
+    <row r="26" ht="80" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Dr. Jennifer Tsuruda</t>
@@ -1920,44 +2200,54 @@
           <t>University of Tennessee, Knoxville</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>https://faculty.utk.edu/Jennifer.Tsuruda</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>Southeast</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>jennifer.tsuruda@utk.edu</t>
         </is>
       </c>
-      <c r="F26" s="2" t="n"/>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>Honey bee health and management, pollination, beekeeper education</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>Runs the TN Master Beekeeping Program (previously at Clemson) - a large existing beekeeper network one door down from NC.</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed — SAS is free system-wide (UTK/UTC/UTHSC/UTM) for faculty, staff, and students, with OIT statistical consulting support.</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J26" s="11" t="n">
+      <c r="L26" s="14" t="n">
         <v>46282</v>
       </c>
-      <c r="K26" s="2" t="n"/>
-      <c r="L26" s="2" t="n"/>
-      <c r="M26" s="2" t="inlineStr">
+      <c r="M26" s="2" t="n"/>
+      <c r="N26" s="2" t="n"/>
+      <c r="O26" s="2" t="inlineStr">
         <is>
           <t>Email inferred from standard UTK firstname.lastname pattern - confirm before sending.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="60" customHeight="1">
+    <row r="27" ht="80" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Dr. Morgan Christman</t>
@@ -1973,40 +2263,50 @@
           <t>LSU AgCenter / Louisiana State University</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>https://www.christmanlab.com/</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>Southeast</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>MChristman@agcenter.lsu.edu</t>
         </is>
       </c>
-      <c r="F27" s="2" t="n"/>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>Pollinator ecology and conservation; building baseline pollinator/native bee data for Louisiana</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>Brand-new program (2025) actively building citizen-science partnerships (a Louisiana Bumble Bee Atlas) - likely receptive to a sister citizen-science project.</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed — SAS 9.4 is available to LSU students/faculty/staff via TigerWare, alongside LSU's Dept. of Experimental Statistics and HPC@LSU computing infrastructure.</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J27" s="11" t="n">
+      <c r="L27" s="14" t="n">
         <v>46231</v>
       </c>
-      <c r="K27" s="2" t="n"/>
-      <c r="L27" s="2" t="n"/>
       <c r="M27" s="2" t="n"/>
-    </row>
-    <row r="28" ht="60" customHeight="1">
+      <c r="N27" s="2" t="n"/>
+      <c r="O27" s="2" t="n"/>
+    </row>
+    <row r="28" ht="80" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Dr. Yong-Lak Park</t>
@@ -2022,48 +2322,58 @@
           <t>West Virginia University</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>https://www.davis.wvu.edu/faculty-staff/directory/yong-lak-park</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>Mid-Atlantic</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Yong-Lak.Park@mail.wvu.edu</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>(304) 293-2882</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>Integrated pest management, pollination ecology of solitary/wild bees, geospatial/remote-sensing methods</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>His geospatial/remote-sensing angle on wild bee ecology is a natural methodological conversation with a location-mapping app.</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed — WVU ITS sells SAS licenses for teaching/non-commercial research through its software store.</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J28" s="11" t="n">
+      <c r="L28" s="14" t="n">
         <v>46287</v>
       </c>
-      <c r="K28" s="2" t="n"/>
-      <c r="L28" s="2" t="n"/>
-      <c r="M28" s="2" t="inlineStr">
+      <c r="M28" s="2" t="n"/>
+      <c r="N28" s="2" t="n"/>
+      <c r="O28" s="2" t="inlineStr">
         <is>
           <t>Focus is broader than honey bees specifically (solitary bees, IPM) - tailor the relevance line accordingly.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="60" customHeight="1">
+    <row r="29" ht="80" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Dr. Rahman Tashakkori</t>
@@ -2079,48 +2389,58 @@
           <t>Appalachian State University</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D29" s="16" t="inlineStr">
+        <is>
+          <t>https://appmais.cs.appstate.edu</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>Southeast</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>tashakkorir@appstate.edu</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>(828) 262-7009</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>Honey bee health monitoring systems (hive sensors, data science, AI) - the AppMAIS/Beemon project</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>Closest technical cousin on this whole list: an NC-based (Boone) honeybee data/monitoring project. Strong potential collaborator, not just an outreach target - worth a more tailored note than the standard boilerplate.</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="J29" s="13" t="inlineStr">
+        <is>
+          <t>Exceptional — App State was one of the first five universities WORLDWIDE to offer courses on the newest SAS Viya platform, and runs a SAS-integrated Business Analytics certificate. Especially fitting for Tashakkori, a CS/data-science PI.</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J29" s="11" t="n">
+      <c r="L29" s="14" t="n">
         <v>46233</v>
       </c>
-      <c r="K29" s="2" t="n"/>
-      <c r="L29" s="2" t="n"/>
-      <c r="M29" s="2" t="inlineStr">
+      <c r="M29" s="2" t="n"/>
+      <c r="N29" s="2" t="n"/>
+      <c r="O29" s="2" t="inlineStr">
         <is>
           <t>Computer Science, not entomology/biology - AppMAIS is the hook, not a traditional bee lab.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="60" customHeight="1">
+    <row r="30" ht="80" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Amy Vu</t>
@@ -2136,45 +2456,55 @@
           <t>University of Florida (Honey Bee Research &amp; Extension Lab)</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D30" s="16" t="inlineStr">
+        <is>
+          <t>https://entnemdept.ufl.edu/people-directory/amy-vu/</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>Southeast</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>amy.vu@ufl.edu</t>
         </is>
       </c>
-      <c r="F30" s="2" t="n"/>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G30" s="2" t="n"/>
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>Beekeeper education, UF Master Beekeeper Program, Bee College, extension outreach</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>Runs UF's beekeeper-facing extension/outreach programs (Bee College, Master Beekeeper Program) - a second, extension-focused UF contact alongside Dr. Ellis's research-focused one.</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed — UF provides free SAS 9.4 access via remote desktop, plus discounted student installs.</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="J30" s="11" t="n">
+      <c r="L30" s="14" t="n">
         <v>46287</v>
       </c>
-      <c r="K30" s="2" t="n"/>
-      <c r="L30" s="2" t="n"/>
-      <c r="M30" s="2" t="inlineStr">
+      <c r="M30" s="2" t="n"/>
+      <c r="N30" s="2" t="n"/>
+      <c r="O30" s="2" t="inlineStr">
         <is>
           <t>Same institution as Jamie Ellis (already on this list) but a distinct extension-facing role - fine to contact both.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M30"/>
+  <autoFilter ref="A1:O30"/>
   <conditionalFormatting sqref="J2:J30">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND(J2&lt;&gt;"",J2&lt;=TODAY())</formula>
@@ -2186,14 +2516,67 @@
       <formula>J2&gt;TODAY()+14</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="K2:K30">
+    <cfRule type="expression" priority="4" dxfId="0">
+      <formula>AND(K2&lt;&gt;"",K2&lt;=TODAY())</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="1">
+      <formula>AND(K2&lt;&gt;"",K2&gt;TODAY(),K2&lt;=TODAY()+14)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="2">
+      <formula>K2&gt;TODAY()+14</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L2:L30">
+    <cfRule type="expression" priority="7" dxfId="0">
+      <formula>AND(L2&lt;&gt;"",L2&lt;=TODAY())</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="1">
+      <formula>AND(L2&lt;&gt;"",L2&gt;TODAY(),L2&lt;=TODAY()+14)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" dxfId="2">
+      <formula>L2&gt;TODAY()+14</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="I2:I30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Contacted,Emailed - Awaiting Reply,Replied,Call/Meeting Scheduled,Declined,No Longer Pursuing,Confirmed - Advisor"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Northeast,Mid-Atlantic,Southeast,Midwest,Great Plains,South Central,Mountain West,Pacific Northwest,West/Pacific"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId29"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2340,10 +2723,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="115" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2379,122 +2762,142 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Column J, Planned Send Date, and what the colors mean:</t>
+          <t>Column D, Department / Lab Link: a clickable link to each contact's faculty profile, lab, or project page — for a quick gut-check on their current work before you email.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>- Blank: already actioned (Tarpy/Delaney/Mahood) or no date set yet.</t>
-        </is>
-      </c>
+      <c r="A8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>- Red/pink: due or overdue — the planned date has arrived or passed and it hasn't been sent.</t>
+          <t>Column J, SAS Software Connection (added Jul 25 2026): since Ronnie's career was at SAS Institute, this flags any public evidence that a contact's university uses SAS software — a natural personal opener ("I spent my career at SAS Institute..."). Green-highlighted 'Exceptional' rows are unusually strong: NC State (SAS was literally founded there in 1966), Clemson ($3.3M SAS gift, renewed through 2026), and Appalachian State (one of the first 5 universities worldwide teaching on SAS Viya). Most others are 'Confirmed' (a standard campus SAS site license, cited). A few are 'Not confirmed' (UC Davis, U Georgia, Michigan State) — no public evidence turned up, so don't assume; ask directly if it's worth knowing before writing that contact.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>- Green: coming up in the next 14 days — a near-term reminder to draft and send.</t>
-        </is>
-      </c>
+      <c r="A10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>- Blue: scheduled further out — no action needed yet.</t>
+          <t>Column K, Planned Send Date, and what the colors mean:</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>These colors update automatically based on today's date each time you open the file.</t>
+          <t>- Blank: already actioned (Tarpy/Delaney/Mahood) or no date set yet.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr"/>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>- Red/pink: due or overdue.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Why the dates are staggered the way they are: 6 contacts are scheduled soon (late Jul - early Aug 2026) because they're less tied to the summer beekeeping field-day calendar — an emeritus researcher (Seeley), a computer-science PI (Tashakkori) whose teaching load is lighter over summer, a brand-new hire actively building partnerships (Christman), a center director (Grozinger), a lab-based researcher (Dolezal), and a data-survey specialist whose busy season is fall/winter (vanEngelsdorp). The other 20 — mostly extension apiculturists running summer field days and Master Beekeeper programs — are staggered after Labor Day (Sept 8, 2026 onward), 3 per day on Tuesdays/Wednesdays/Thursdays, to avoid a mass-blast pattern and land in inboxes when they're actually checking email regularly.</t>
+          <t>- Green: coming up in the next 14 days.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr"/>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>- Blue: scheduled further out.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>How to use this sheet:</t>
+          <t>Colors update automatically based on today's date each time the file opens.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>1. Update the Status dropdown (column I) as you email each contact: Not Contacted -&gt; Emailed - Awaiting Reply -&gt; Replied / Call-Meeting Scheduled / Declined / No Longer Pursuing / Confirmed - Advisor.</t>
-        </is>
-      </c>
+      <c r="A17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2. Adjust Planned Send Date (column J) any time — drag rows around, push dates out, whatever fits.</t>
+          <t>Why the dates are staggered the way they are: 6 contacts are scheduled soon (late Jul - early Aug 2026) because they're less tied to the summer beekeeping field-day calendar. The other 20 — mostly extension apiculturists running summer field days — are staggered after Labor Day (Sept 8, 2026 onward), 3 per day on Tuesdays/Wednesdays/Thursdays.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>3. Fill in Date Emailed (column K) when you actually send.</t>
-        </is>
-      </c>
+      <c r="A19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>4. Set a Follow-up Date (column L) — 2-3 weeks after sending is a reasonable default if there's no reply.</t>
+          <t>How to use this sheet:</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>5. Use Notes (column M) for anything short and specific.</t>
+          <t>1. Update the Status dropdown (column K) as you email each contact.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>6. US Region (column D) is a dropdown too, in case you add more contacts later and want the categories to stay consistent.</t>
+          <t>2. Adjust Planned Send Date (column L) any time.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr"/>
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>3. Fill in Date Emailed (column M) when you actually send.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Batches so far: Already-in-motion (4, Jul 25 2026) — Seeley, Tarpy, Delaney, Mahood. Batch 1 (19, Jul 25 2026) — national spread. Batch 2 (6, Jul 25 2026) — Southeast-focused. 29 contacts total.</t>
+          <t>4. Set a Follow-up Date (column N) — 2-3 weeks after sending is a reasonable default.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr"/>
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>5. Use Notes (column O) for anything short and specific.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>6. US Region (column E) is a dropdown too, in case you add more contacts later.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Batches so far: Already-in-motion (4, Jul 25 2026) — Seeley, Tarpy, Delaney, Mahood. Batch 1 (19, Jul 25 2026) — national spread. Batch 2 (6, Jul 25 2026) — Southeast-focused. 29 contacts total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>This list is separate from KEY_PEOPLE_CONTACTS.md in the project repo. Once outreach starts, it's worth mirroring status updates into that file too so both stay in sync.</t>
         </is>

</xml_diff>

<commit_message>
Revise email template opening with SAS Institute personal connection
</commit_message>
<xml_diff>
--- a/University_Bee_Research_Contacts.xlsx
+++ b/University_Bee_Research_Contacts.xlsx
@@ -120,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -160,6 +160,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2587,7 +2590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2601,6 +2604,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -2608,13 +2612,14 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1">
+    <row r="4" ht="70" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Copy the Subject and Body below into Gmail for each contact. Fill in the bracketed placeholders using that contact's row on the "University Contacts" tab — Name, Institution, and especially the "Why Relevant to SaveTheHives" column, which is written so it can drop almost directly into [RELEVANCE SENTENCE]. Keep the rest as-is; it's deliberately short. After sending, update Status and Date Emailed on the University Contacts tab.</t>
-        </is>
-      </c>
-    </row>
+          <t>Copy the Subject and Body below into Gmail for each contact. Fill in the bracketed placeholders using that contact's row on the "University Contacts" tab — Name, Institution, the "Why Relevant" column (drops almost directly into [RELEVANCE SENTENCE]), and the "SAS Software Connection" column (drops into [SAS CONNECTION SENTENCE] — see note below). Keep the rest as-is; it's deliberately short. After sending, update Status and Date Emailed on the University Contacts tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
@@ -2622,7 +2627,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="20" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t>[FIRST NAME]</t>
@@ -2634,7 +2639,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="20" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>[LAST NAME]</t>
@@ -2646,7 +2651,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="20" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>[INSTITUTION]</t>
@@ -2658,44 +2663,63 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="60" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
+          <t>[SAS CONNECTION SENTENCE]</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Optional, one line, only if the SAS Software Connection column has something. For 'Exceptional' rows (NC State, Clemson, Appalachian State) lean into the specific fact — e.g. "Funny enough, SAS actually got its start just down the road at NC State, so this feels like a bit of a small-world moment." For 'Confirmed' rows, something lighter — e.g. "I noticed [INSTITUTION] runs SAS for some of its research computing, which made writing this feel a little less like a cold email." For 'Not confirmed' or 'N/A' rows, delete this sentence entirely rather than guessing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
           <t>[RELEVANCE SENTENCE]</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>One sentence tying their specific research to SaveTheHives — start from the "Why Relevant" column and adjust the wording so it reads naturally in a sentence.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="4" t="n"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Subject</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Wild honeybee colony mapping project — thought of your work at [INSTITUTION]</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="4" t="n"/>
+    </row>
+    <row r="16" ht="430" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Body</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="430" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+    <row r="17" ht="460" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Hi Dr. [LAST NAME],
-My name is Ronnie Bouchon, and I run SaveTheHives (savethehives.org), a free citizen-science app for mapping wild/feral honeybee colonies — tree cavities, structures, ground nests, wherever people find them. The app currently has 1,150+ historical hive records live on the map (many concentrated around the NC Triangle), and volunteers can log new colonies or simply re-verify ("Validate") an existing one.
+My name is Ronnie Bouchon. I'm a retired beekeeper who spent most of my career in data and analytics, mostly at SAS Institute — and now that I'm retired, I've been putting that background to use on something closer to home: SaveTheHives (savethehives.org), a free citizen-science app for mapping wild/feral honeybee colonies — tree cavities, structures, ground nests, wherever people find them. [SAS CONNECTION SENTENCE]
+The app currently has 1,150+ historical hive records live on the map (many concentrated around the NC Triangle), and volunteers can log new colonies or simply re-verify ("Validate") an existing one.
 The core idea is tracking colony resilience: hives that survive 3+ winters untreated are strong candidates for heritable Varroa resistance — we've been calling them "Genetic Goldmines." Dr. David Tarpy at NC State reviewed and approved that framing and is a named scientific advisor on the project.
 [RELEVANCE SENTENCE]
 I'm not asking for anything formal — just wanted to put SaveTheHives on your radar. If it's useful to you, your students, or your extension audience as a way to crowdsource wild colony locations in your region, I'd genuinely appreciate you sharing it or pointing people our way. Happy to answer questions or hop on a quick call if that's ever useful.
@@ -2709,9 +2733,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A14:B14"/>
     <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A17:B17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Revise send-date timing by career stage; add Career Stage/Timing Rationale column
Per Dr. Tarpy's comment that he no longer does much personal fieldwork and
is now funding/mentoring-focused, reviewed all 26 not-yet-contacted university
contacts by role. Moved 6 senior PI/Center-Director/Emeritus contacts (Spivak,
Ellis, Hopkins, McArt, Delaplane, Williams) from September to Aug 11-20 since
they aren't tied to a summer field-day calendar. Left true Extension
specialists/agents (who do run summer field days) in the fall batch, and left
early-career researchers unchanged. Added column P documenting the rationale
per contact, and a revision note on the How to Use tab.
</commit_message>
<xml_diff>
--- a/University_Bee_Research_Contacts.xlsx
+++ b/University_Bee_Research_Contacts.xlsx
@@ -556,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O30"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -574,6 +574,7 @@
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="34" customWidth="1" min="15" max="15"/>
+    <col width="55" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -652,6 +653,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Career Stage / Timing Rationale</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -717,6 +723,11 @@
       <c r="O2" s="9" t="inlineStr">
         <is>
           <t>Extremely high-value contact - worth a personally written email referencing the 2015 Apidologie paper rather than the generic boilerplate.</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>Emeritus — no active lab or field-day calendar; timing not field-driven.</t>
         </is>
       </c>
     </row>
@@ -780,6 +791,11 @@
           <t>Already actively engaged - not part of the cold-outreach batches below. Included here so this list reads as complete when shared with him. See MEETING_NOTES_2026-07-21_Tarpy.md for full context.</t>
         </is>
       </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed advisor; senior — per his own comment, now funding/mentoring-focused rather than fieldwork. Already in motion.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="9" t="inlineStr">
@@ -849,6 +865,11 @@
           <t>Reintroduction email sent 2026-07-25 (see delaney-email.html / KEY_PEOPLE_CONTACTS.md). Not part of the cold-outreach batches below - included here so this list reads as complete when shared with Tarpy.</t>
         </is>
       </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>Senior endowed professor — funding/program focus, not field-day bound. Already emailed.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
@@ -912,6 +933,11 @@
       <c r="O5" s="9" t="inlineStr">
         <is>
           <t>Sent via mapmydca.com/contact-us/ (no personal email published) - date is approximate/session date, correct if off. See KEY_PEOPLE_CONTACTS.md.</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>Independent citizen-scientist, not academic — no field-day calendar applies. Already emailed.</t>
         </is>
       </c>
     </row>
@@ -977,6 +1003,11 @@
       <c r="M6" s="2" t="n"/>
       <c r="N6" s="2" t="n"/>
       <c r="O6" s="2" t="n"/>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>Center Director — grant/program-focused, not field-day bound. Moved earlier (was Sept, now Aug).</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="80" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -1035,7 +1066,7 @@
         </is>
       </c>
       <c r="L7" s="14" t="n">
-        <v>46273</v>
+        <v>46245</v>
       </c>
       <c r="M7" s="2" t="n"/>
       <c r="N7" s="2" t="n"/>
@@ -1044,6 +1075,11 @@
           <t>Emeritus - personal email not published; route through lab contact form or department (entomology@umn.edu).</t>
         </is>
       </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>Emeritus — no active lab/field-day calendar. Moved earlier (was Sept, now Aug).</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="80" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -1107,6 +1143,11 @@
       <c r="M8" s="2" t="n"/>
       <c r="N8" s="2" t="n"/>
       <c r="O8" s="2" t="n"/>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>Cooperative Extension specialist — runs summer field days for beekeepers. Fall timing holds.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="80" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -1170,6 +1211,11 @@
       <c r="M9" s="2" t="n"/>
       <c r="N9" s="2" t="n"/>
       <c r="O9" s="2" t="n"/>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>Associate Professor, hands-on research program — likely active in field/lab over summer. Timing unchanged.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="80" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -1228,11 +1274,16 @@
         </is>
       </c>
       <c r="L10" s="14" t="n">
-        <v>46274</v>
+        <v>46246</v>
       </c>
       <c r="M10" s="2" t="n"/>
       <c r="N10" s="2" t="n"/>
       <c r="O10" s="2" t="n"/>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>Lab Director — grant/oversight-focused, not field-day bound. Moved earlier (was Sept, now Aug).</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="80" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -1287,7 +1338,7 @@
         </is>
       </c>
       <c r="L11" s="14" t="n">
-        <v>46274</v>
+        <v>46247</v>
       </c>
       <c r="M11" s="2" t="n"/>
       <c r="N11" s="2" t="n"/>
@@ -1296,6 +1347,11 @@
           <t>Succeeded Steve Sheppard (retired 2024) as program lead.</t>
         </is>
       </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>Distinguished Professor, senior — program-focused. Moved earlier (was Sept, now Aug).</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="80" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -1359,6 +1415,11 @@
       <c r="M12" s="2" t="n"/>
       <c r="N12" s="2" t="n"/>
       <c r="O12" s="2" t="n"/>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>Associate Professor, hands-on lab research. Timing unchanged.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="80" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
@@ -1413,7 +1474,7 @@
         </is>
       </c>
       <c r="L13" s="14" t="n">
-        <v>46275</v>
+        <v>46252</v>
       </c>
       <c r="M13" s="2" t="n"/>
       <c r="N13" s="2" t="n"/>
@@ -1422,6 +1483,11 @@
           <t>General lab inbox is dycelab@cornell.edu if personal email bounces.</t>
         </is>
       </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>Lab Director — grant/oversight-focused, not field-day bound. Moved earlier (was Sept, now Aug).</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="80" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -1480,11 +1546,16 @@
         </is>
       </c>
       <c r="L14" s="14" t="n">
-        <v>46275</v>
+        <v>46253</v>
       </c>
       <c r="M14" s="2" t="n"/>
       <c r="N14" s="2" t="n"/>
       <c r="O14" s="2" t="n"/>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>Emeritus + Program Director — no personal field-day calendar. Moved earlier (was Sept, now Aug).</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="80" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -1543,11 +1614,16 @@
         </is>
       </c>
       <c r="L15" s="14" t="n">
-        <v>46275</v>
+        <v>46254</v>
       </c>
       <c r="M15" s="2" t="n"/>
       <c r="N15" s="2" t="n"/>
       <c r="O15" s="2" t="n"/>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>Center Director — grant/program-focused, not field-day bound. Moved earlier (was Sept, now Aug).</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="80" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -1615,6 +1691,11 @@
           <t>Email inferred from standard OSU firstname.lastname pattern - confirm before sending (site lists it as an obfuscated mailto).</t>
         </is>
       </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>Extension apiculturist — runs summer field days. Fall timing holds.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="80" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
@@ -1682,6 +1763,11 @@
           <t>Strong candidate to lead with - his own work is citizen-science-adjacent.</t>
         </is>
       </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>Chief Scientist, Bee Informed Partnership — coordination/data role, not field-day bound. Already scheduled early.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="80" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -1745,6 +1831,11 @@
       <c r="M18" s="2" t="n"/>
       <c r="N18" s="2" t="n"/>
       <c r="O18" s="2" t="n"/>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>Extension specialist, breeding program — hands-on summer field work. Fall timing holds.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="80" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
@@ -1812,6 +1903,11 @@
           <t>Lab inbox shown; address email to Dr. Milbrath by name.</t>
         </is>
       </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>Extension coordinator — runs trainings/field days. Fall timing holds.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="80" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -1875,6 +1971,11 @@
       <c r="M20" s="2" t="n"/>
       <c r="N20" s="2" t="n"/>
       <c r="O20" s="2" t="n"/>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>Extension specialist — summer field days. Fall timing holds.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="80" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
@@ -1938,6 +2039,11 @@
       <c r="M21" s="2" t="n"/>
       <c r="N21" s="2" t="n"/>
       <c r="O21" s="2" t="n"/>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>Associate Professor, lab-based research — already scheduled early, no change needed.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="80" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -2001,6 +2107,11 @@
       <c r="M22" s="2" t="n"/>
       <c r="N22" s="2" t="n"/>
       <c r="O22" s="2" t="n"/>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>Full professor, hands-on research program. Timing unchanged.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="80" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
@@ -2064,6 +2175,11 @@
       <c r="M23" s="2" t="n"/>
       <c r="N23" s="2" t="n"/>
       <c r="O23" s="2" t="n"/>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>Associate Professor, hands-on lab research. Timing unchanged.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="80" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -2123,6 +2239,11 @@
       <c r="M24" s="2" t="n"/>
       <c r="N24" s="2" t="n"/>
       <c r="O24" s="2" t="n"/>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>Associate Professor, hands-on research. Timing unchanged.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="80" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
@@ -2186,6 +2307,11 @@
       <c r="M25" s="2" t="n"/>
       <c r="N25" s="2" t="n"/>
       <c r="O25" s="2" t="n"/>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>Extension coordinator — summer field days. Fall timing holds.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="80" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -2249,6 +2375,11 @@
           <t>Email inferred from standard UTK firstname.lastname pattern - confirm before sending.</t>
         </is>
       </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>Assistant Professor + Extension specialist — hands-on/field-day heavy. Timing unchanged.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="80" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
@@ -2308,6 +2439,11 @@
       <c r="M27" s="2" t="n"/>
       <c r="N27" s="2" t="n"/>
       <c r="O27" s="2" t="n"/>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>Assistant Professor, brand-new program — hands-on herself. Already scheduled early, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="80" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
@@ -2375,6 +2511,11 @@
           <t>Focus is broader than honey bees specifically (solitary bees, IPM) - tailor the relevance line accordingly.</t>
         </is>
       </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>Full professor, geospatial/tech-leaning research — lower field-day dependence, not urgent to move.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="80" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
@@ -2442,6 +2583,11 @@
           <t>Computer Science, not entomology/biology - AppMAIS is the hook, not a traditional bee lab.</t>
         </is>
       </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>CS professor, tech/data project (AppMAIS) — not bee-fieldwork bound at all. Already scheduled early.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="80" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
@@ -2503,6 +2649,11 @@
       <c r="O30" s="2" t="inlineStr">
         <is>
           <t>Same institution as Jamie Ellis (already on this list) but a distinct extension-facing role - fine to contact both.</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>Extension agent — runs Bee College/field days. Fall timing holds.</t>
         </is>
       </c>
     </row>
@@ -2604,7 +2755,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -2619,7 +2769,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
@@ -2747,7 +2896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -2927,6 +3076,51 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Revision (Jul 25 2026 follow-up): Ronnie relayed that Dr. Tarpy told him he no longer does much personal fieldwork — his role now is growing projects, securing funding, and mentoring undergrad/grad students who do the hands-on work. That prompted a review of the whole list by career stage:</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>- True Extension specialists/agents/coordinators (Nino, Sagili, Harris, Vu, Powell, Given, Milbrath, Tsuruda) genuinely run summer field days — fall timing was kept for these.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>- Senior PIs who are now Center/Lab Directors, plus Emeritus faculty (Grozinger, Ellis, Hopkins, McArt, Delaplane, Williams, Spivak) are grant/program-focused like Tarpy described, not tied to a field-day calendar — moved from Sept to Aug 11-20, 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>- Early-career researchers building their own labs (Rangel, Johnson, Dolezal, Joshi, Wu-Smart, Couvillon, Christman) are likely still hands-on themselves — timing left unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>- Non-apiculture contacts (Tashakkori, a CS professor running a hive-tech project) aren't tied to a bee field-day calendar at all — already scheduled early.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>See new column P, 'Career Stage / Timing Rationale', for the specific reasoning per contact.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add personalized outreach lines; document SAS sync workflow
</commit_message>
<xml_diff>
--- a/University_Bee_Research_Contacts.xlsx
+++ b/University_Bee_Research_Contacts.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'University Contacts'!$A$1:$O$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'University Contacts'!$A$1:$R$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -68,7 +68,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -91,6 +91,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D9EAD3"/>
         <bgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE5CD"/>
+        <bgColor rgb="00FCE5CD"/>
       </patternFill>
     </fill>
   </fills>
@@ -120,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -163,6 +169,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -556,25 +565,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P30"/>
+  <dimension ref="A1:R30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="34" customWidth="1" min="15" max="15"/>
-    <col width="55" customWidth="1" min="16" max="16"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="34" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -625,41 +636,51 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Personalized Relevance Sentence (drafted)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>SAS Software Connection</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Personalized SAS Sentence (drafted)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Planned Send Date</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Date Emailed</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Follow-up Date</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Career Stage / Timing Rationale</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="90" customHeight="1">
+    <row r="2" ht="100" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
           <t>Dr. Thomas D. Seeley</t>
@@ -707,31 +728,41 @@
       </c>
       <c r="J2" s="9" t="inlineStr">
         <is>
+          <t>Your Arnot Forest work is honestly the reason SaveTheHives frames long-surviving wild colonies as "Genetic Goldmines" in the first place - we're hoping the app can help surface more real-world examples of exactly the kind of untreated, Varroa-adapted colonies you've studied there for decades, and it doesn't hurt that David Tarpy and Debbie Delaney, both already involved with the project, are co-authors with you on the 2015 Apidologie survivor-colony paper.</t>
+        </is>
+      </c>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
           <t>Confirmed — Cornell IT holds a campus-wide SAS site license (Base/SAS, SAS/STAT, Enterprise Guide, etc.) available to faculty, staff, and students.</t>
         </is>
       </c>
-      <c r="K2" s="9" t="inlineStr">
+      <c r="L2" s="9" t="inlineStr">
+        <is>
+          <t>I noticed Cornell runs a campus-wide SAS license too, which made writing this feel a little less like a cold email.</t>
+        </is>
+      </c>
+      <c r="M2" s="9" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L2" s="12" t="n">
+      <c r="N2" s="12" t="n">
         <v>46232</v>
       </c>
-      <c r="M2" s="9" t="n"/>
-      <c r="N2" s="9" t="n"/>
-      <c r="O2" s="9" t="inlineStr">
+      <c r="O2" s="9" t="n"/>
+      <c r="P2" s="9" t="n"/>
+      <c r="Q2" s="9" t="inlineStr">
         <is>
           <t>Extremely high-value contact - worth a personally written email referencing the 2015 Apidologie paper rather than the generic boilerplate.</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="R2" s="9" t="inlineStr">
         <is>
           <t>Emeritus — no active lab or field-day calendar; timing not field-driven.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="90" customHeight="1">
+    <row r="3" ht="100" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Dr. David R. Tarpy</t>
@@ -773,31 +804,33 @@
           <t>Named scientific advisor on SaveTheHives' 'Genetic Goldmine' framing since the Jul 21 2026 lunch meeting - reviewed and approved all 5 questions on the language handout. Helped get the original savethehives.com press coverage in 2008.</t>
         </is>
       </c>
-      <c r="J3" s="9" t="inlineStr">
+      <c r="J3" s="9" t="inlineStr"/>
+      <c r="K3" s="9" t="inlineStr">
         <is>
           <t>Exceptional — SAS Institute was literally founded at NC State (1966) as an agricultural-data research project - Jim Goodnight and colleagues built the original SAS there before spinning it out in 1976. SAS Hall (math/stats building) is named for the founders, and SAS still actively partners with NC State's Plant Sciences Initiative. Hard to beat as a personal connection.</t>
         </is>
       </c>
-      <c r="K3" s="9" t="inlineStr">
+      <c r="L3" s="9" t="inlineStr"/>
+      <c r="M3" s="9" t="inlineStr">
         <is>
           <t>Confirmed - Advisor</t>
         </is>
       </c>
-      <c r="L3" s="9" t="n"/>
-      <c r="M3" s="9" t="n"/>
       <c r="N3" s="9" t="n"/>
-      <c r="O3" s="9" t="inlineStr">
+      <c r="O3" s="9" t="n"/>
+      <c r="P3" s="9" t="n"/>
+      <c r="Q3" s="9" t="inlineStr">
         <is>
           <t>Already actively engaged - not part of the cold-outreach batches below. Included here so this list reads as complete when shared with him. See MEETING_NOTES_2026-07-21_Tarpy.md for full context.</t>
         </is>
       </c>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="R3" s="9" t="inlineStr">
         <is>
           <t>Confirmed advisor; senior — per his own comment, now funding/mentoring-focused rather than fieldwork. Already in motion.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="90" customHeight="1">
+    <row r="4" ht="100" customHeight="1">
       <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Dr. Debbie Delaney</t>
@@ -843,35 +876,37 @@
           <t>Her UD faculty page lists savethehives.com as one of her own resource links - she was directly involved with the original 2008-era project alongside Tarpy. Co-author with Tarpy and Seeley on the 2015 Apidologie survivor-colony genetics paper - directly on-thesis for the Genetic Goldmine framing.</t>
         </is>
       </c>
-      <c r="J4" s="9" t="inlineStr">
+      <c r="J4" s="9" t="inlineStr"/>
+      <c r="K4" s="9" t="inlineStr">
         <is>
           <t>Confirmed — UD licenses SAS for teaching and research (annual license via UDeploy), sub-licensable by departments.</t>
         </is>
       </c>
-      <c r="K4" s="9" t="inlineStr">
+      <c r="L4" s="9" t="inlineStr"/>
+      <c r="M4" s="9" t="inlineStr">
         <is>
           <t>Emailed - Awaiting Reply</t>
-        </is>
-      </c>
-      <c r="L4" s="9" t="n"/>
-      <c r="M4" s="9" t="inlineStr">
-        <is>
-          <t>2026-07-25</t>
         </is>
       </c>
       <c r="N4" s="9" t="n"/>
       <c r="O4" s="9" t="inlineStr">
         <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="P4" s="9" t="n"/>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
           <t>Reintroduction email sent 2026-07-25 (see delaney-email.html / KEY_PEOPLE_CONTACTS.md). Not part of the cold-outreach batches below - included here so this list reads as complete when shared with Tarpy.</t>
         </is>
       </c>
-      <c r="P4" s="2" t="inlineStr">
+      <c r="R4" s="9" t="inlineStr">
         <is>
           <t>Senior endowed professor — funding/program focus, not field-day bound. Already emailed.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="90" customHeight="1">
+    <row r="5" ht="100" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Julia Mahood</t>
@@ -913,35 +948,37 @@
           <t>Very close citizen-science cousin to SaveTheHives - the app already has a 'DCA Mapping' feature marked 'coming soon.' 2018 Georgia Beekeeper of the Year; guest on Beekeeping Today and OSU Extension's PolliNation podcasts.</t>
         </is>
       </c>
-      <c r="J5" s="9" t="inlineStr">
+      <c r="J5" s="9" t="inlineStr"/>
+      <c r="K5" s="9" t="inlineStr">
         <is>
           <t>Not researched</t>
         </is>
       </c>
-      <c r="K5" s="9" t="inlineStr">
+      <c r="L5" s="9" t="inlineStr"/>
+      <c r="M5" s="9" t="inlineStr">
         <is>
           <t>Emailed - Awaiting Reply</t>
-        </is>
-      </c>
-      <c r="L5" s="9" t="n"/>
-      <c r="M5" s="9" t="inlineStr">
-        <is>
-          <t>2026-07-25</t>
         </is>
       </c>
       <c r="N5" s="9" t="n"/>
       <c r="O5" s="9" t="inlineStr">
         <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="P5" s="9" t="n"/>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
           <t>Sent via mapmydca.com/contact-us/ (no personal email published) - date is approximate/session date, correct if off. See KEY_PEOPLE_CONTACTS.md.</t>
         </is>
       </c>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="R5" s="9" t="inlineStr">
         <is>
           <t>Independent citizen-scientist, not academic — no field-day calendar applies. Already emailed.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="80" customHeight="1">
+    <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Dr. Christina Grozinger</t>
@@ -987,29 +1024,39 @@
           <t>Directs one of the largest pollinator research centers in the US, with a strong extension/outreach arm that could amplify a citizen-science mapping project.</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>With the Center for Pollinator Research running some of the country's most active extension and public-outreach programs, I'm hoping SaveTheHives might be a useful citizen-science tool to point your audience toward, or simply something worth having on your radar.</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>Confirmed — Penn State distributes SAS 9.4 licenses to faculty/staff/students through its Software Store, renewed annually.</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>I noticed Penn State runs SAS through its Software Store as well, which made writing this feel a little less like a cold email.</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="N6" s="14" t="n">
         <v>46239</v>
       </c>
-      <c r="M6" s="2" t="n"/>
-      <c r="N6" s="2" t="n"/>
       <c r="O6" s="2" t="n"/>
-      <c r="P6" s="2" t="inlineStr">
+      <c r="P6" s="2" t="n"/>
+      <c r="Q6" s="2" t="n"/>
+      <c r="R6" s="2" t="inlineStr">
         <is>
           <t>Center Director — grant/program-focused, not field-day bound. Moved earlier (was Sept, now Aug).</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="80" customHeight="1">
+    <row r="7" ht="90" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Dr. Marla Spivak</t>
@@ -1055,33 +1102,35 @@
           <t>The 'Genetic Goldmine' framing (survivor colonies bred for resistance) is essentially her life's work; a major name if she engages, even briefly.</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Confirmed — SAS is licensed campus-wide through IT@UMN for teaching, learning, and research.</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L7" s="14" t="n">
+      <c r="N7" s="14" t="n">
         <v>46245</v>
       </c>
-      <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="n"/>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="O7" s="2" t="n"/>
+      <c r="P7" s="2" t="n"/>
+      <c r="Q7" s="2" t="inlineStr">
         <is>
           <t>Emeritus - personal email not published; route through lab contact form or department (entomology@umn.edu).</t>
         </is>
       </c>
-      <c r="P7" s="2" t="inlineStr">
+      <c r="R7" s="2" t="inlineStr">
         <is>
           <t>Emeritus — no active lab/field-day calendar. Moved earlier (was Sept, now Aug).</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="80" customHeight="1">
+    <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Dr. Elina Nino</t>
@@ -1127,29 +1176,31 @@
           <t>West Coast counterpart to NC State's program; UC Davis runs one of the country's top honey bee research facilities.</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Not confirmed — UC Davis's Computational Research Service prominently licenses SPSS; no clear public SAS-specific site license page turned up in search. Worth asking Dr. Niño directly rather than assuming.</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L8" s="14" t="n">
+      <c r="N8" s="14" t="n">
         <v>46273</v>
       </c>
-      <c r="M8" s="2" t="n"/>
-      <c r="N8" s="2" t="n"/>
       <c r="O8" s="2" t="n"/>
-      <c r="P8" s="2" t="inlineStr">
+      <c r="P8" s="2" t="n"/>
+      <c r="Q8" s="2" t="n"/>
+      <c r="R8" s="2" t="inlineStr">
         <is>
           <t>Cooperative Extension specialist — runs summer field days for beekeepers. Fall timing holds.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="80" customHeight="1">
+    <row r="9" ht="90" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Dr. Juliana Rangel</t>
@@ -1195,29 +1246,31 @@
           <t>Leads a major state bee program in a region with a strong feral/Africanized colony research thread already in our contact notes.</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>Confirmed — SAS is available through the Texas A&amp;M Software Center and is used directly in the Statistics department's curriculum.</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L9" s="14" t="n">
+      <c r="N9" s="14" t="n">
         <v>46273</v>
       </c>
-      <c r="M9" s="2" t="n"/>
-      <c r="N9" s="2" t="n"/>
       <c r="O9" s="2" t="n"/>
-      <c r="P9" s="2" t="inlineStr">
+      <c r="P9" s="2" t="n"/>
+      <c r="Q9" s="2" t="n"/>
+      <c r="R9" s="2" t="inlineStr">
         <is>
           <t>Associate Professor, hands-on research program — likely active in field/lab over summer. Timing unchanged.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="80" customHeight="1">
+    <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Dr. Jamie Ellis</t>
@@ -1263,29 +1316,31 @@
           <t>HBREL runs active feral-colony removal and trapping research - closely adjacent to SaveTheHives' core mapping mission.</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Confirmed — UF provides free SAS 9.4 access via remote desktop, plus discounted student installs.</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L10" s="14" t="n">
+      <c r="N10" s="14" t="n">
         <v>46246</v>
       </c>
-      <c r="M10" s="2" t="n"/>
-      <c r="N10" s="2" t="n"/>
       <c r="O10" s="2" t="n"/>
-      <c r="P10" s="2" t="inlineStr">
+      <c r="P10" s="2" t="n"/>
+      <c r="Q10" s="2" t="n"/>
+      <c r="R10" s="2" t="inlineStr">
         <is>
           <t>Lab Director — grant/oversight-focused, not field-day bound. Moved earlier (was Sept, now Aug).</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="80" customHeight="1">
+    <row r="11" ht="90" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Dr. Brandon Hopkins</t>
@@ -1327,33 +1382,35 @@
           <t>Genetic-diversity/germplasm preservation work lines up directly with the 'Genetic Goldmine' survivor-genetics framing.</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Confirmed — SAS is available via WSU's Software Site License, with CAHNRS (the ag college) specifically licensing it for Biological Systems Engineering.</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L11" s="14" t="n">
+      <c r="N11" s="14" t="n">
         <v>46247</v>
       </c>
-      <c r="M11" s="2" t="n"/>
-      <c r="N11" s="2" t="n"/>
-      <c r="O11" s="2" t="inlineStr">
+      <c r="O11" s="2" t="n"/>
+      <c r="P11" s="2" t="n"/>
+      <c r="Q11" s="2" t="inlineStr">
         <is>
           <t>Succeeded Steve Sheppard (retired 2024) as program lead.</t>
         </is>
       </c>
-      <c r="P11" s="2" t="inlineStr">
+      <c r="R11" s="2" t="inlineStr">
         <is>
           <t>Distinguished Professor, senior — program-focused. Moved earlier (was Sept, now Aug).</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="80" customHeight="1">
+    <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Dr. Reed Johnson</t>
@@ -1399,29 +1456,31 @@
           <t>Strong Midwest program with an active beekeeper-facing extension arm.</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>Confirmed — Ohio State licenses both Teaching/Research and Administrative versions of SAS campus-wide, renewed each September; the Statistics department actively supports it.</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L12" s="14" t="n">
+      <c r="N12" s="14" t="n">
         <v>46274</v>
       </c>
-      <c r="M12" s="2" t="n"/>
-      <c r="N12" s="2" t="n"/>
       <c r="O12" s="2" t="n"/>
-      <c r="P12" s="2" t="inlineStr">
+      <c r="P12" s="2" t="n"/>
+      <c r="Q12" s="2" t="n"/>
+      <c r="R12" s="2" t="inlineStr">
         <is>
           <t>Associate Professor, hands-on lab research. Timing unchanged.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="80" customHeight="1">
+    <row r="13" ht="90" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Dr. Scott McArt</t>
@@ -1463,33 +1522,35 @@
           <t>Northeast counterpart to Tarpy's NC State program; Dyce Lab has a large beekeeper-facing extension program to cross-promote with.</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>Confirmed — Cornell IT holds a campus-wide SAS site license (Base/SAS, SAS/STAT, Enterprise Guide, etc.) available to faculty, staff, and students.</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L13" s="14" t="n">
+      <c r="N13" s="14" t="n">
         <v>46252</v>
       </c>
-      <c r="M13" s="2" t="n"/>
-      <c r="N13" s="2" t="n"/>
-      <c r="O13" s="2" t="inlineStr">
+      <c r="O13" s="2" t="n"/>
+      <c r="P13" s="2" t="n"/>
+      <c r="Q13" s="2" t="inlineStr">
         <is>
           <t>General lab inbox is dycelab@cornell.edu if personal email bounces.</t>
         </is>
       </c>
-      <c r="P13" s="2" t="inlineStr">
+      <c r="R13" s="2" t="inlineStr">
         <is>
           <t>Lab Director — grant/oversight-focused, not field-day bound. Moved earlier (was Sept, now Aug).</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="80" customHeight="1">
+    <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Dr. Keith Delaplane</t>
@@ -1535,29 +1596,31 @@
           <t>Adjacent Southeast state; UGA runs a large Master Beekeeper Program that could help cross-promote SaveTheHives.</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>Not confirmed — Found SAS access via special Data Services workstations in the library, but no clear campus-wide site license page. Worth asking Delaplane directly rather than assuming.</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L14" s="14" t="n">
+      <c r="N14" s="14" t="n">
         <v>46253</v>
       </c>
-      <c r="M14" s="2" t="n"/>
-      <c r="N14" s="2" t="n"/>
       <c r="O14" s="2" t="n"/>
-      <c r="P14" s="2" t="inlineStr">
+      <c r="P14" s="2" t="n"/>
+      <c r="Q14" s="2" t="n"/>
+      <c r="R14" s="2" t="inlineStr">
         <is>
           <t>Emeritus + Program Director — no personal field-day calendar. Moved earlier (was Sept, now Aug).</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="80" customHeight="1">
+    <row r="15" ht="90" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Dr. Geoff Williams</t>
@@ -1603,29 +1666,31 @@
           <t>Adjacent Southeast state with a growing, well-funded bee center.</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>Confirmed — Auburn's College of Agriculture runs a dedicated 'SAS and R Statistical Software Resources' page - directly relevant since Williams is in that college.</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L15" s="14" t="n">
+      <c r="N15" s="14" t="n">
         <v>46254</v>
       </c>
-      <c r="M15" s="2" t="n"/>
-      <c r="N15" s="2" t="n"/>
       <c r="O15" s="2" t="n"/>
-      <c r="P15" s="2" t="inlineStr">
+      <c r="P15" s="2" t="n"/>
+      <c r="Q15" s="2" t="n"/>
+      <c r="R15" s="2" t="inlineStr">
         <is>
           <t>Center Director — grant/program-focused, not field-day bound. Moved earlier (was Sept, now Aug).</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="80" customHeight="1">
+    <row r="16" ht="90" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Dr. Ramesh Sagili</t>
@@ -1671,33 +1736,35 @@
           <t>West Coast program with an active Master Beekeeper Program and strong grower/beekeeper outreach.</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>Confirmed — OSU participates in a campus-wide SAS site license; College of Forestry has its own block of 75 licenses.</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L16" s="14" t="n">
+      <c r="N16" s="14" t="n">
         <v>46280</v>
       </c>
-      <c r="M16" s="2" t="n"/>
-      <c r="N16" s="2" t="n"/>
-      <c r="O16" s="2" t="inlineStr">
+      <c r="O16" s="2" t="n"/>
+      <c r="P16" s="2" t="n"/>
+      <c r="Q16" s="2" t="inlineStr">
         <is>
           <t>Email inferred from standard OSU firstname.lastname pattern - confirm before sending (site lists it as an obfuscated mailto).</t>
         </is>
       </c>
-      <c r="P16" s="2" t="inlineStr">
+      <c r="R16" s="2" t="inlineStr">
         <is>
           <t>Extension apiculturist — runs summer field days. Fall timing holds.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="80" customHeight="1">
+    <row r="17" ht="90" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Dr. Dennis vanEngelsdorp</t>
@@ -1743,33 +1810,43 @@
           <t>Runs the country's largest citizen-science bee health survey (the annual national Colony Loss Survey) - the closest methodological cousin to SaveTheHives on this list.</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J17" s="18" t="inlineStr">
+        <is>
+          <t>Your Bee Informed Partnership colony-loss survey is the closest thing I know of to what SaveTheHives is trying to do at a smaller scale - crowdsourced, on-the-ground data on how colonies are actually faring - so I'd love your take on whether the two could be useful to each other.</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>Confirmed — UMD DivIT sells and renews SAS licenses for teaching/research use.</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="L17" s="18" t="inlineStr">
+        <is>
+          <t>I also noticed Maryland licenses SAS through DivIT, which made writing this feel a little less like a cold email.</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L17" s="14" t="n">
+      <c r="N17" s="14" t="n">
         <v>46238</v>
       </c>
-      <c r="M17" s="2" t="n"/>
-      <c r="N17" s="2" t="n"/>
-      <c r="O17" s="2" t="inlineStr">
+      <c r="O17" s="2" t="n"/>
+      <c r="P17" s="2" t="n"/>
+      <c r="Q17" s="2" t="inlineStr">
         <is>
           <t>Strong candidate to lead with - his own work is citizen-science-adjacent.</t>
         </is>
       </c>
-      <c r="P17" s="2" t="inlineStr">
+      <c r="R17" s="2" t="inlineStr">
         <is>
           <t>Chief Scientist, Bee Informed Partnership — coordination/data role, not field-day bound. Already scheduled early.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="80" customHeight="1">
+    <row r="18" ht="90" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Krispn Given</t>
@@ -1815,29 +1892,31 @@
           <t>Directly on-thesis: breeding survivor stock for Varroa resistance.</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>Confirmed — SAS is available through Purdue's Research Computing (RCAC) and supported by the Statistics department's free consulting service.</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L18" s="14" t="n">
+      <c r="N18" s="14" t="n">
         <v>46280</v>
       </c>
-      <c r="M18" s="2" t="n"/>
-      <c r="N18" s="2" t="n"/>
       <c r="O18" s="2" t="n"/>
-      <c r="P18" s="2" t="inlineStr">
+      <c r="P18" s="2" t="n"/>
+      <c r="Q18" s="2" t="n"/>
+      <c r="R18" s="2" t="inlineStr">
         <is>
           <t>Extension specialist, breeding program — hands-on summer field work. Fall timing holds.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="80" customHeight="1">
+    <row r="19" ht="90" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Dr. Meghan Milbrath</t>
@@ -1883,33 +1962,35 @@
           <t>Trains veterinary students/professionals in honey bee medicine - an outreach channel beyond the typical beekeeping audience.</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>Not confirmed — Search kept surfacing University of Michigan instead of MSU; no clear MSU-specific SAS site license page found. Worth asking Milbrath directly rather than assuming.</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L19" s="14" t="n">
+      <c r="N19" s="14" t="n">
         <v>46280</v>
       </c>
-      <c r="M19" s="2" t="n"/>
-      <c r="N19" s="2" t="n"/>
-      <c r="O19" s="2" t="inlineStr">
+      <c r="O19" s="2" t="n"/>
+      <c r="P19" s="2" t="n"/>
+      <c r="Q19" s="2" t="inlineStr">
         <is>
           <t>Lab inbox shown; address email to Dr. Milbrath by name.</t>
         </is>
       </c>
-      <c r="P19" s="2" t="inlineStr">
+      <c r="R19" s="2" t="inlineStr">
         <is>
           <t>Extension coordinator — runs trainings/field days. Fall timing holds.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="80" customHeight="1">
+    <row r="20" ht="90" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Dr. Jeff Harris</t>
@@ -1955,29 +2036,31 @@
           <t>Deep South program with a breeding focus that aligns closely with the Genetic Goldmine framing.</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>Confirmed — MSU holds a limited campus site license for SAS, with public access via the Mitchell Memorial Library Computer Commons.</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L20" s="14" t="n">
+      <c r="N20" s="14" t="n">
         <v>46281</v>
       </c>
-      <c r="M20" s="2" t="n"/>
-      <c r="N20" s="2" t="n"/>
       <c r="O20" s="2" t="n"/>
-      <c r="P20" s="2" t="inlineStr">
+      <c r="P20" s="2" t="n"/>
+      <c r="Q20" s="2" t="n"/>
+      <c r="R20" s="2" t="inlineStr">
         <is>
           <t>Extension specialist — summer field days. Fall timing holds.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="80" customHeight="1">
+    <row r="21" ht="90" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Dr. Adam Dolezal</t>
@@ -2023,29 +2106,39 @@
           <t>Studies wild-managed bee interactions directly relevant to feral colony tracking.</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J21" s="18" t="inlineStr">
+        <is>
+          <t>Since your lab studies how managed and wild bees interact and pass along stress and disease, I thought the feral colony location data SaveTheHives is collecting might eventually be a useful resource for exactly that kind of research.</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>Confirmed — SAS Education Analytical Suite is distributed campus-wide via the Illinois WebStore.</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="L21" s="18" t="inlineStr">
+        <is>
+          <t>I noticed Illinois distributes SAS campus-wide too, which made writing this feel a little less like a cold email.</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L21" s="14" t="n">
+      <c r="N21" s="14" t="n">
         <v>46240</v>
       </c>
-      <c r="M21" s="2" t="n"/>
-      <c r="N21" s="2" t="n"/>
       <c r="O21" s="2" t="n"/>
-      <c r="P21" s="2" t="inlineStr">
+      <c r="P21" s="2" t="n"/>
+      <c r="Q21" s="2" t="n"/>
+      <c r="R21" s="2" t="inlineStr">
         <is>
           <t>Associate Professor, lab-based research — already scheduled early, no change needed.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="80" customHeight="1">
+    <row r="22" ht="90" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Dr. Neelendra Joshi</t>
@@ -2091,29 +2184,31 @@
           <t>Fills a south-central US research gap in this list.</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>Confirmed — SAS site licenses are free for faculty and students, distributed via sitelicense.uark.edu.</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L22" s="14" t="n">
+      <c r="N22" s="14" t="n">
         <v>46281</v>
       </c>
-      <c r="M22" s="2" t="n"/>
-      <c r="N22" s="2" t="n"/>
       <c r="O22" s="2" t="n"/>
-      <c r="P22" s="2" t="inlineStr">
+      <c r="P22" s="2" t="n"/>
+      <c r="Q22" s="2" t="n"/>
+      <c r="R22" s="2" t="inlineStr">
         <is>
           <t>Full professor, hands-on research program. Timing unchanged.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="80" customHeight="1">
+    <row r="23" ht="90" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Dr. Judy Wu-Smart</t>
@@ -2159,29 +2254,31 @@
           <t>Great Plains program; trained under Marla Spivak, a nice connective thread if both are contacted.</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>Confirmed — UNL struck a new no-cost enterprise-wide SAS agreement in Oct 2024, and hosts an active local Nebraska SAS Users Group (NEBSUG) for training/networking.</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L23" s="14" t="n">
+      <c r="N23" s="14" t="n">
         <v>46281</v>
       </c>
-      <c r="M23" s="2" t="n"/>
-      <c r="N23" s="2" t="n"/>
       <c r="O23" s="2" t="n"/>
-      <c r="P23" s="2" t="inlineStr">
+      <c r="P23" s="2" t="n"/>
+      <c r="Q23" s="2" t="n"/>
+      <c r="R23" s="2" t="inlineStr">
         <is>
           <t>Associate Professor, hands-on lab research. Timing unchanged.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="80" customHeight="1">
+    <row r="24" ht="90" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Dr. Margaret Couvillon</t>
@@ -2223,29 +2320,31 @@
           <t>Adjacent to NC/VA; foraging-ecology research could make direct use of SaveTheHives' colony location data.</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>Confirmed — SAS is available via VT Software Distribution, and VT's Statistical Applications and Innovation Group (SAIG) supports it directly.</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L24" s="14" t="n">
+      <c r="N24" s="14" t="n">
         <v>46282</v>
       </c>
-      <c r="M24" s="2" t="n"/>
-      <c r="N24" s="2" t="n"/>
       <c r="O24" s="2" t="n"/>
-      <c r="P24" s="2" t="inlineStr">
+      <c r="P24" s="2" t="n"/>
+      <c r="Q24" s="2" t="n"/>
+      <c r="R24" s="2" t="inlineStr">
         <is>
           <t>Associate Professor, hands-on research. Timing unchanged.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="80" customHeight="1">
+    <row r="25" ht="90" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
           <t>Ben Powell</t>
@@ -2291,29 +2390,31 @@
           <t>Neighboring state extension program (SC) with an active beekeeper-facing newsletter (CAPPings) that could carry a SaveTheHives mention statewide.</t>
         </is>
       </c>
-      <c r="J25" s="13" t="inlineStr">
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="13" t="inlineStr">
         <is>
           <t>Exceptional — SAS gifted Clemson $3.3M in software licensing (2021, renewed through 2026) covering Base SAS and cloud-based SAS Viya for ~25,000 users, specifically to power big-data/analytics research and teaching.</t>
         </is>
       </c>
-      <c r="K25" s="2" t="inlineStr">
+      <c r="L25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L25" s="14" t="n">
+      <c r="N25" s="14" t="n">
         <v>46282</v>
       </c>
-      <c r="M25" s="2" t="n"/>
-      <c r="N25" s="2" t="n"/>
       <c r="O25" s="2" t="n"/>
-      <c r="P25" s="2" t="inlineStr">
+      <c r="P25" s="2" t="n"/>
+      <c r="Q25" s="2" t="n"/>
+      <c r="R25" s="2" t="inlineStr">
         <is>
           <t>Extension coordinator — summer field days. Fall timing holds.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="80" customHeight="1">
+    <row r="26" ht="90" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Dr. Jennifer Tsuruda</t>
@@ -2355,33 +2456,35 @@
           <t>Runs the TN Master Beekeeping Program (previously at Clemson) - a large existing beekeeper network one door down from NC.</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>Confirmed — SAS is free system-wide (UTK/UTC/UTHSC/UTM) for faculty, staff, and students, with OIT statistical consulting support.</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L26" s="14" t="n">
+      <c r="N26" s="14" t="n">
         <v>46282</v>
       </c>
-      <c r="M26" s="2" t="n"/>
-      <c r="N26" s="2" t="n"/>
-      <c r="O26" s="2" t="inlineStr">
+      <c r="O26" s="2" t="n"/>
+      <c r="P26" s="2" t="n"/>
+      <c r="Q26" s="2" t="inlineStr">
         <is>
           <t>Email inferred from standard UTK firstname.lastname pattern - confirm before sending.</t>
         </is>
       </c>
-      <c r="P26" s="2" t="inlineStr">
+      <c r="R26" s="2" t="inlineStr">
         <is>
           <t>Assistant Professor + Extension specialist — hands-on/field-day heavy. Timing unchanged.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="80" customHeight="1">
+    <row r="27" ht="90" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Dr. Morgan Christman</t>
@@ -2423,29 +2526,39 @@
           <t>Brand-new program (2025) actively building citizen-science partnerships (a Louisiana Bumble Bee Atlas) - likely receptive to a sister citizen-science project.</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="J27" s="18" t="inlineStr">
+        <is>
+          <t>I saw you're building out a Louisiana Bumble Bee Atlas with citizen scientists, and it sounds like exactly the kind of project SaveTheHives is trying to be for wild honeybee colonies - would love to compare notes on what's worked for getting volunteers to actually contribute good data.</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>Confirmed — SAS 9.4 is available to LSU students/faculty/staff via TigerWare, alongside LSU's Dept. of Experimental Statistics and HPC@LSU computing infrastructure.</t>
         </is>
       </c>
-      <c r="K27" s="2" t="inlineStr">
+      <c r="L27" s="18" t="inlineStr">
+        <is>
+          <t>I also noticed LSU makes SAS available to students and faculty through TigerWare, which made writing this feel a little less like a cold email.</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L27" s="14" t="n">
+      <c r="N27" s="14" t="n">
         <v>46231</v>
       </c>
-      <c r="M27" s="2" t="n"/>
-      <c r="N27" s="2" t="n"/>
       <c r="O27" s="2" t="n"/>
-      <c r="P27" s="2" t="inlineStr">
+      <c r="P27" s="2" t="n"/>
+      <c r="Q27" s="2" t="n"/>
+      <c r="R27" s="2" t="inlineStr">
         <is>
           <t>Assistant Professor, brand-new program — hands-on herself. Already scheduled early, no change.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="80" customHeight="1">
+    <row r="28" ht="90" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Dr. Yong-Lak Park</t>
@@ -2491,33 +2604,35 @@
           <t>His geospatial/remote-sensing angle on wild bee ecology is a natural methodological conversation with a location-mapping app.</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>Confirmed — WVU ITS sells SAS licenses for teaching/non-commercial research through its software store.</t>
         </is>
       </c>
-      <c r="K28" s="2" t="inlineStr">
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L28" s="14" t="n">
+      <c r="N28" s="14" t="n">
         <v>46287</v>
       </c>
-      <c r="M28" s="2" t="n"/>
-      <c r="N28" s="2" t="n"/>
-      <c r="O28" s="2" t="inlineStr">
+      <c r="O28" s="2" t="n"/>
+      <c r="P28" s="2" t="n"/>
+      <c r="Q28" s="2" t="inlineStr">
         <is>
           <t>Focus is broader than honey bees specifically (solitary bees, IPM) - tailor the relevance line accordingly.</t>
         </is>
       </c>
-      <c r="P28" s="2" t="inlineStr">
+      <c r="R28" s="2" t="inlineStr">
         <is>
           <t>Full professor, geospatial/tech-leaning research — lower field-day dependence, not urgent to move.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="80" customHeight="1">
+    <row r="29" ht="90" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Dr. Rahman Tashakkori</t>
@@ -2563,33 +2678,43 @@
           <t>Closest technical cousin on this whole list: an NC-based (Boone) honeybee data/monitoring project. Strong potential collaborator, not just an outreach target - worth a more tailored note than the standard boilerplate.</t>
         </is>
       </c>
-      <c r="J29" s="13" t="inlineStr">
+      <c r="J29" s="18" t="inlineStr">
+        <is>
+          <t>AppMAIS looks like the closest thing to a technical sibling that SaveTheHives has - you're monitoring hive health with sensors and data science, we're crowdsourcing hive locations and survival data, and both projects are trying to get better information about colonies that aren't in a beekeeper's backyard. Would love to hear if there's ever a way the two could talk to each other, even informally.</t>
+        </is>
+      </c>
+      <c r="K29" s="13" t="inlineStr">
         <is>
           <t>Exceptional — App State was one of the first five universities WORLDWIDE to offer courses on the newest SAS Viya platform, and runs a SAS-integrated Business Analytics certificate. Especially fitting for Tashakkori, a CS/data-science PI.</t>
         </is>
       </c>
-      <c r="K29" s="2" t="inlineStr">
+      <c r="L29" s="18" t="inlineStr">
+        <is>
+          <t>Funny enough, I noticed App State was one of the first five universities anywhere teaching on SAS's newest Viya platform - SAS was basically my whole career, so that felt like a nice bit of overlap.</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L29" s="14" t="n">
+      <c r="N29" s="14" t="n">
         <v>46233</v>
       </c>
-      <c r="M29" s="2" t="n"/>
-      <c r="N29" s="2" t="n"/>
-      <c r="O29" s="2" t="inlineStr">
+      <c r="O29" s="2" t="n"/>
+      <c r="P29" s="2" t="n"/>
+      <c r="Q29" s="2" t="inlineStr">
         <is>
           <t>Computer Science, not entomology/biology - AppMAIS is the hook, not a traditional bee lab.</t>
         </is>
       </c>
-      <c r="P29" s="2" t="inlineStr">
+      <c r="R29" s="2" t="inlineStr">
         <is>
           <t>CS professor, tech/data project (AppMAIS) — not bee-fieldwork bound at all. Already scheduled early.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="80" customHeight="1">
+    <row r="30" ht="90" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Amy Vu</t>
@@ -2631,34 +2756,36 @@
           <t>Runs UF's beekeeper-facing extension/outreach programs (Bee College, Master Beekeeper Program) - a second, extension-focused UF contact alongside Dr. Ellis's research-focused one.</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr">
         <is>
           <t>Confirmed — UF provides free SAS 9.4 access via remote desktop, plus discounted student installs.</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr">
+      <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr">
         <is>
           <t>Not Contacted</t>
         </is>
       </c>
-      <c r="L30" s="14" t="n">
+      <c r="N30" s="14" t="n">
         <v>46287</v>
       </c>
-      <c r="M30" s="2" t="n"/>
-      <c r="N30" s="2" t="n"/>
-      <c r="O30" s="2" t="inlineStr">
+      <c r="O30" s="2" t="n"/>
+      <c r="P30" s="2" t="n"/>
+      <c r="Q30" s="2" t="inlineStr">
         <is>
           <t>Same institution as Jamie Ellis (already on this list) but a distinct extension-facing role - fine to contact both.</t>
         </is>
       </c>
-      <c r="P30" s="2" t="inlineStr">
+      <c r="R30" s="2" t="inlineStr">
         <is>
           <t>Extension agent — runs Bee College/field days. Fall timing holds.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O30"/>
+  <autoFilter ref="A1:R30"/>
   <conditionalFormatting sqref="J2:J30">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND(J2&lt;&gt;"",J2&lt;=TODAY())</formula>
@@ -2692,8 +2819,19 @@
       <formula>L2&gt;TODAY()+14</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="N2:N30">
+    <cfRule type="expression" priority="10" dxfId="0">
+      <formula>AND(N2&lt;&gt;"",N2&lt;=TODAY())</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" dxfId="1">
+      <formula>AND(N2&lt;&gt;"",N2&gt;TODAY(),N2&lt;=TODAY()+14)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" dxfId="2">
+      <formula>N2&gt;TODAY()+14</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="K2:K30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Contacted,Emailed - Awaiting Reply,Replied,Call/Meeting Scheduled,Declined,No Longer Pursuing,Confirmed - Advisor"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -2925,7 +3063,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Rows 2-5 (highlighted tan): Dr. Thomas Seeley (Cornell), Dr. David Tarpy (NC State), Dr. Debbie Delaney (U Delaware), and Julia Mahood (Map My DCA, Atlanta) — contacts already central to or already in motion for this project, listed first so the sheet reads as complete at a glance if shared with Tarpy.</t>
+          <t>Rows 2-5 (tan): Seeley, Tarpy, Delaney, Mahood — already central to or already in motion for this project.</t>
         </is>
       </c>
     </row>
@@ -2935,7 +3073,7 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Column D, Department / Lab Link: a clickable link to each contact's faculty profile, lab, or project page — for a quick gut-check on their current work before you email.</t>
+          <t>Columns J and L (orange fill where filled in), added Jul 26 2026: Personalized Relevance Sentence and Personalized SAS Sentence — ready-to-paste replacements for the [RELEVANCE SENTENCE] and [SAS CONNECTION SENTENCE] placeholders on the Email Template tab. Drafted so far for the 6 contacts going out soonest: Seeley, Christman, Tashakkori, vanEngelsdorp, Grozinger, Dolezal. Blank for everyone else — draft theirs the same way (pull from the Why Relevant / SAS Software Connection columns, write it in first person as Ronnie) as their Planned Send Date approaches.</t>
         </is>
       </c>
     </row>
@@ -2945,7 +3083,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Column J, SAS Software Connection (added Jul 25 2026): since Ronnie's career was at SAS Institute, this flags any public evidence that a contact's university uses SAS software — a natural personal opener ("I spent my career at SAS Institute..."). Green-highlighted 'Exceptional' rows are unusually strong: NC State (SAS was literally founded there in 1966), Clemson ($3.3M SAS gift, renewed through 2026), and Appalachian State (one of the first 5 universities worldwide teaching on SAS Viya). Most others are 'Confirmed' (a standard campus SAS site license, cited). A few are 'Not confirmed' (UC Davis, U Georgia, Michigan State) — no public evidence turned up, so don't assume; ask directly if it's worth knowing before writing that contact.</t>
+          <t>Column K, SAS Software Connection: 'Exceptional' rows (green fill) get a specific, named fact in the personalized sentence (e.g. Tashakkori/App State's SAS Viya program). 'Confirmed' rows get a lighter, one-line mention. 'Not confirmed' or 'N/A' rows should have that sentence deleted entirely from the email, not guessed at.</t>
         </is>
       </c>
     </row>
@@ -2955,14 +3093,14 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Column K, Planned Send Date, and what the colors mean:</t>
+          <t>Column N, Planned Send Date, and what the colors mean:</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>- Blank: already actioned (Tarpy/Delaney/Mahood) or no date set yet.</t>
+          <t>- Blank: already actioned or no date set.</t>
         </is>
       </c>
     </row>
@@ -3000,126 +3138,95 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Why the dates are staggered the way they are: 6 contacts are scheduled soon (late Jul - early Aug 2026) because they're less tied to the summer beekeeping field-day calendar. The other 20 — mostly extension apiculturists running summer field days — are staggered after Labor Day (Sept 8, 2026 onward), 3 per day on Tuesdays/Wednesdays/Thursdays.</t>
+          <t>How to use this sheet:</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr"/>
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>1. When a contact's Planned Send Date turns green, draft their Personalized Relevance Sentence and SAS Sentence (columns J and L) if not already done.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>How to use this sheet:</t>
+          <t>2. Copy the Email Template tab's Subject/Body into Gmail, swap in [FIRST NAME], [LAST NAME], [INSTITUTION], and the two drafted sentences.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>1. Update the Status dropdown (column K) as you email each contact.</t>
+          <t>3. Update Status (column M) and Date Emailed (column O) once sent.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2. Adjust Planned Send Date (column L) any time.</t>
+          <t>4. Set a Follow-up Date (column P) — 2-3 weeks out is a reasonable default.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>3. Fill in Date Emailed (column M) when you actually send.</t>
+          <t>5. Use Notes (column Q) for anything short and specific.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>4. Set a Follow-up Date (column N) — 2-3 weeks after sending is a reasonable default.</t>
-        </is>
-      </c>
+      <c r="A24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>5. Use Notes (column O) for anything short and specific.</t>
+          <t>Batches so far: Already-in-motion (4, Jul 25) — Seeley, Tarpy, Delaney, Mahood. Batch 1 (19, Jul 25) — national spread. Batch 2 (6, Jul 25) — Southeast-focused. 29 contacts total. Personalized lines drafted for the first 6 going out (Jul 26).</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>6. US Region (column E) is a dropdown too, in case you add more contacts later.</t>
-        </is>
-      </c>
+      <c r="A26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="inlineStr"/>
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>This list is separate from KEY_PEOPLE_CONTACTS.md in the project repo. Mirror status updates there too so both stay in sync.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>Batches so far: Already-in-motion (4, Jul 25 2026) — Seeley, Tarpy, Delaney, Mahood. Batch 1 (19, Jul 25 2026) — national spread. Batch 2 (6, Jul 25 2026) — Southeast-focused. 29 contacts total.</t>
-        </is>
-      </c>
+      <c r="A28" s="5" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr"/>
+      <c r="A29" s="5" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>This list is separate from KEY_PEOPLE_CONTACTS.md in the project repo. Once outreach starts, it's worth mirroring status updates into that file too so both stay in sync.</t>
-        </is>
-      </c>
-    </row>
+      <c r="A30" s="5" t="n"/>
+    </row>
+    <row r="31"/>
     <row r="32">
-      <c r="A32" s="5" t="inlineStr"/>
+      <c r="A32" s="5" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>Revision (Jul 25 2026 follow-up): Ronnie relayed that Dr. Tarpy told him he no longer does much personal fieldwork — his role now is growing projects, securing funding, and mentoring undergrad/grad students who do the hands-on work. That prompted a review of the whole list by career stage:</t>
-        </is>
-      </c>
+      <c r="A33" s="5" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>- True Extension specialists/agents/coordinators (Nino, Sagili, Harris, Vu, Powell, Given, Milbrath, Tsuruda) genuinely run summer field days — fall timing was kept for these.</t>
-        </is>
-      </c>
+      <c r="A34" s="5" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>- Senior PIs who are now Center/Lab Directors, plus Emeritus faculty (Grozinger, Ellis, Hopkins, McArt, Delaplane, Williams, Spivak) are grant/program-focused like Tarpy described, not tied to a field-day calendar — moved from Sept to Aug 11-20, 2026.</t>
-        </is>
-      </c>
+      <c r="A35" s="5" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>- Early-career researchers building their own labs (Rangel, Johnson, Dolezal, Joshi, Wu-Smart, Couvillon, Christman) are likely still hands-on themselves — timing left unchanged.</t>
-        </is>
-      </c>
+      <c r="A36" s="5" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>- Non-apiculture contacts (Tashakkori, a CS professor running a hive-tech project) aren't tied to a bee field-day calendar at all — already scheduled early.</t>
-        </is>
-      </c>
+      <c r="A37" s="5" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="inlineStr">
-        <is>
-          <t>See new column P, 'Career Stage / Timing Rationale', for the specific reasoning per contact.</t>
-        </is>
-      </c>
+      <c r="A38" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix Date Emailed color-suppression rule on Planned Send Date; remove stale CF cruft
</commit_message>
<xml_diff>
--- a/University_Bee_Research_Contacts.xlsx
+++ b/University_Bee_Research_Contacts.xlsx
@@ -2786,47 +2786,17 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:R30"/>
-  <conditionalFormatting sqref="J2:J30">
-    <cfRule type="expression" priority="1" dxfId="0">
-      <formula>AND(J2&lt;&gt;"",J2&lt;=TODAY())</formula>
+  <conditionalFormatting sqref="N2:N30">
+    <cfRule type="expression" priority="1" stopIfTrue="1">
+      <formula>O2&lt;&gt;""</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1">
-      <formula>AND(J2&lt;&gt;"",J2&gt;TODAY(),J2&lt;=TODAY()+14)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="3" dxfId="2">
-      <formula>J2&gt;TODAY()+14</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K30">
-    <cfRule type="expression" priority="4" dxfId="0">
-      <formula>AND(K2&lt;&gt;"",K2&lt;=TODAY())</formula>
-    </cfRule>
-    <cfRule type="expression" priority="5" dxfId="1">
-      <formula>AND(K2&lt;&gt;"",K2&gt;TODAY(),K2&lt;=TODAY()+14)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="6" dxfId="2">
-      <formula>K2&gt;TODAY()+14</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L2:L30">
-    <cfRule type="expression" priority="7" dxfId="0">
-      <formula>AND(L2&lt;&gt;"",L2&lt;=TODAY())</formula>
-    </cfRule>
-    <cfRule type="expression" priority="8" dxfId="1">
-      <formula>AND(L2&lt;&gt;"",L2&gt;TODAY(),L2&lt;=TODAY()+14)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="9" dxfId="2">
-      <formula>L2&gt;TODAY()+14</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N2:N30">
-    <cfRule type="expression" priority="10" dxfId="0">
+    <cfRule type="expression" priority="2" dxfId="0">
       <formula>AND(N2&lt;&gt;"",N2&lt;=TODAY())</formula>
     </cfRule>
-    <cfRule type="expression" priority="11" dxfId="1">
+    <cfRule type="expression" priority="3" dxfId="1">
       <formula>AND(N2&lt;&gt;"",N2&gt;TODAY(),N2&lt;=TODAY()+14)</formula>
     </cfRule>
-    <cfRule type="expression" priority="12" dxfId="2">
+    <cfRule type="expression" priority="4" dxfId="2">
       <formula>N2&gt;TODAY()+14</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3206,7 +3176,6 @@
     <row r="30">
       <c r="A30" s="5" t="n"/>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="5" t="n"/>
     </row>

</xml_diff>